<commit_message>
Enhanced formula to handle complex sheet
</commit_message>
<xml_diff>
--- a/thaco/Office-1.xlsx
+++ b/thaco/Office-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adity/Documents/GitHub/gitlocal/thaco/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3715331D-91B2-4540-B968-5BFEE1D4AB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37514C91-9D22-9445-9B85-42FFEA3BAD17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38800" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="761" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="761" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bảng lương CB-NV" sheetId="1" r:id="rId1"/>
@@ -4286,16 +4286,71 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
+            <color rgb="FF000000"/>
             <rFont val="Calibri"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
-          <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    TV: Thử việc
-CT: Chính thức</t>
+          <t xml:space="preserve">[Threaded comment]
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Comment:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">    TV: Thử việc
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t>CT: Chính thức</t>
         </r>
       </text>
     </comment>
@@ -4304,18 +4359,91 @@
         <r>
           <rPr>
             <sz val="11"/>
-            <color theme="1"/>
+            <color rgb="FF000000"/>
             <rFont val="Calibri"/>
             <family val="2"/>
-            <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Đối tượng Lương ngày tại các TĐTV
-Reply:
-    LT: Lương Tháng
-LN: Lương ngày
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Comment:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">    Đối tượng Lương ngày tại các TĐTV
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Reply:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">    LT: Lương Tháng
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">LN: Lương ngày
 </t>
         </r>
       </text>
@@ -4417,7 +4545,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="156">
   <si>
     <t>COMPANY …..............</t>
   </si>
@@ -4897,6 +5025,12 @@
   <si>
     <t>Description of Salary Advance Sheet - Period 1</t>
   </si>
+  <si>
+    <t>Description of Employee Payroll</t>
+  </si>
+  <si>
+    <t>Description of Period 1 Advance Payroll</t>
+  </si>
 </sst>
 </file>
 
@@ -4909,7 +5043,7 @@
     <numFmt numFmtId="166" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="59">
+  <fonts count="62">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5288,6 +5422,24 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF3B3B3B"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.4"/>
+      <color rgb="FF374151"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9.4"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -5590,7 +5742,7 @@
     <xf numFmtId="0" fontId="46" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="46" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="301">
+  <cellXfs count="304">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -6253,23 +6405,90 @@
     <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="58" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="28" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="22" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="27" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="24" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="22" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="27" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="28" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="28" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -6279,8 +6498,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -6288,116 +6505,54 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="18" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="22" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="24" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="165" fontId="22" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="22" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="22" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="43" fontId="22" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="27" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="18" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="22" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="23" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="58" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="59" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="61" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="9">
     <cellStyle name="1991-" xfId="3" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
@@ -7164,88 +7319,88 @@
       <c r="CD2" s="12"/>
     </row>
     <row r="3" spans="1:87" s="16" customFormat="1" ht="24" customHeight="1" outlineLevel="1">
-      <c r="A3" s="277"/>
-      <c r="B3" s="274"/>
-      <c r="C3" s="274"/>
-      <c r="D3" s="274"/>
-      <c r="E3" s="274"/>
-      <c r="F3" s="274"/>
-      <c r="G3" s="274"/>
-      <c r="H3" s="274"/>
-      <c r="I3" s="274"/>
-      <c r="J3" s="274"/>
-      <c r="K3" s="274"/>
-      <c r="L3" s="274"/>
-      <c r="M3" s="274"/>
-      <c r="N3" s="274"/>
-      <c r="O3" s="274"/>
-      <c r="P3" s="274"/>
-      <c r="Q3" s="274"/>
-      <c r="R3" s="274"/>
-      <c r="S3" s="274"/>
-      <c r="T3" s="274"/>
-      <c r="U3" s="274"/>
-      <c r="V3" s="274"/>
-      <c r="W3" s="274"/>
-      <c r="X3" s="274"/>
-      <c r="Y3" s="274"/>
-      <c r="Z3" s="274"/>
-      <c r="AA3" s="274"/>
-      <c r="AB3" s="274"/>
-      <c r="AC3" s="274"/>
-      <c r="AD3" s="274"/>
-      <c r="AE3" s="274"/>
-      <c r="AF3" s="274"/>
-      <c r="AG3" s="274"/>
-      <c r="AH3" s="274"/>
-      <c r="AI3" s="274"/>
-      <c r="AJ3" s="274"/>
-      <c r="AK3" s="274"/>
-      <c r="AL3" s="274"/>
-      <c r="AM3" s="274"/>
-      <c r="AN3" s="274"/>
-      <c r="AO3" s="274"/>
-      <c r="AP3" s="274"/>
-      <c r="AQ3" s="274"/>
-      <c r="AR3" s="274"/>
-      <c r="AS3" s="274"/>
-      <c r="AT3" s="274"/>
-      <c r="AU3" s="274"/>
-      <c r="AV3" s="274"/>
-      <c r="AW3" s="274"/>
-      <c r="AX3" s="274"/>
-      <c r="AY3" s="274"/>
-      <c r="AZ3" s="274"/>
-      <c r="BA3" s="274"/>
-      <c r="BB3" s="274"/>
-      <c r="BC3" s="274"/>
-      <c r="BD3" s="274"/>
-      <c r="BE3" s="274"/>
-      <c r="BF3" s="274"/>
-      <c r="BG3" s="274"/>
-      <c r="BH3" s="274"/>
-      <c r="BI3" s="274"/>
-      <c r="BJ3" s="274"/>
-      <c r="BK3" s="274"/>
-      <c r="BL3" s="274"/>
-      <c r="BM3" s="274"/>
-      <c r="BN3" s="274"/>
-      <c r="BO3" s="274"/>
-      <c r="BP3" s="274"/>
-      <c r="BQ3" s="274"/>
-      <c r="BR3" s="274"/>
-      <c r="BS3" s="274"/>
-      <c r="BT3" s="274"/>
-      <c r="BU3" s="274"/>
+      <c r="A3" s="268"/>
+      <c r="B3" s="266"/>
+      <c r="C3" s="266"/>
+      <c r="D3" s="266"/>
+      <c r="E3" s="266"/>
+      <c r="F3" s="266"/>
+      <c r="G3" s="266"/>
+      <c r="H3" s="266"/>
+      <c r="I3" s="266"/>
+      <c r="J3" s="266"/>
+      <c r="K3" s="266"/>
+      <c r="L3" s="266"/>
+      <c r="M3" s="266"/>
+      <c r="N3" s="266"/>
+      <c r="O3" s="266"/>
+      <c r="P3" s="266"/>
+      <c r="Q3" s="266"/>
+      <c r="R3" s="266"/>
+      <c r="S3" s="266"/>
+      <c r="T3" s="266"/>
+      <c r="U3" s="266"/>
+      <c r="V3" s="266"/>
+      <c r="W3" s="266"/>
+      <c r="X3" s="266"/>
+      <c r="Y3" s="266"/>
+      <c r="Z3" s="266"/>
+      <c r="AA3" s="266"/>
+      <c r="AB3" s="266"/>
+      <c r="AC3" s="266"/>
+      <c r="AD3" s="266"/>
+      <c r="AE3" s="266"/>
+      <c r="AF3" s="266"/>
+      <c r="AG3" s="266"/>
+      <c r="AH3" s="266"/>
+      <c r="AI3" s="266"/>
+      <c r="AJ3" s="266"/>
+      <c r="AK3" s="266"/>
+      <c r="AL3" s="266"/>
+      <c r="AM3" s="266"/>
+      <c r="AN3" s="266"/>
+      <c r="AO3" s="266"/>
+      <c r="AP3" s="266"/>
+      <c r="AQ3" s="266"/>
+      <c r="AR3" s="266"/>
+      <c r="AS3" s="266"/>
+      <c r="AT3" s="266"/>
+      <c r="AU3" s="266"/>
+      <c r="AV3" s="266"/>
+      <c r="AW3" s="266"/>
+      <c r="AX3" s="266"/>
+      <c r="AY3" s="266"/>
+      <c r="AZ3" s="266"/>
+      <c r="BA3" s="266"/>
+      <c r="BB3" s="266"/>
+      <c r="BC3" s="266"/>
+      <c r="BD3" s="266"/>
+      <c r="BE3" s="266"/>
+      <c r="BF3" s="266"/>
+      <c r="BG3" s="266"/>
+      <c r="BH3" s="266"/>
+      <c r="BI3" s="266"/>
+      <c r="BJ3" s="266"/>
+      <c r="BK3" s="266"/>
+      <c r="BL3" s="266"/>
+      <c r="BM3" s="266"/>
+      <c r="BN3" s="266"/>
+      <c r="BO3" s="266"/>
+      <c r="BP3" s="266"/>
+      <c r="BQ3" s="266"/>
+      <c r="BR3" s="266"/>
+      <c r="BS3" s="266"/>
+      <c r="BT3" s="266"/>
+      <c r="BU3" s="266"/>
       <c r="BV3" s="110"/>
-      <c r="BW3" s="273" t="s">
+      <c r="BW3" s="265" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="274"/>
-      <c r="BY3" s="274"/>
-      <c r="BZ3" s="274"/>
-      <c r="CA3" s="274"/>
-      <c r="CB3" s="274"/>
+      <c r="BX3" s="266"/>
+      <c r="BY3" s="266"/>
+      <c r="BZ3" s="266"/>
+      <c r="CA3" s="266"/>
+      <c r="CB3" s="266"/>
       <c r="CC3" s="71"/>
       <c r="CD3" s="71"/>
       <c r="CE3" s="240" t="s">
@@ -7329,12 +7484,12 @@
       <c r="BT4" s="15"/>
       <c r="BU4" s="15"/>
       <c r="BV4" s="111"/>
-      <c r="BW4" s="274"/>
-      <c r="BX4" s="274"/>
-      <c r="BY4" s="274"/>
-      <c r="BZ4" s="274"/>
-      <c r="CA4" s="274"/>
-      <c r="CB4" s="274"/>
+      <c r="BW4" s="266"/>
+      <c r="BX4" s="266"/>
+      <c r="BY4" s="266"/>
+      <c r="BZ4" s="266"/>
+      <c r="CA4" s="266"/>
+      <c r="CB4" s="266"/>
       <c r="CC4" s="71"/>
       <c r="CD4" s="71"/>
     </row>
@@ -7412,12 +7567,12 @@
       <c r="BT5" s="15"/>
       <c r="BU5" s="15"/>
       <c r="BV5" s="111"/>
-      <c r="BW5" s="275"/>
-      <c r="BX5" s="275"/>
-      <c r="BY5" s="275"/>
-      <c r="BZ5" s="275"/>
-      <c r="CA5" s="275"/>
-      <c r="CB5" s="275"/>
+      <c r="BW5" s="267"/>
+      <c r="BX5" s="267"/>
+      <c r="BY5" s="267"/>
+      <c r="BZ5" s="267"/>
+      <c r="CA5" s="267"/>
+      <c r="CB5" s="267"/>
       <c r="CC5" s="71"/>
       <c r="CD5" s="71"/>
     </row>
@@ -7495,12 +7650,12 @@
       <c r="BT6" s="18"/>
       <c r="BU6" s="18"/>
       <c r="BV6" s="112"/>
-      <c r="BW6" s="275"/>
-      <c r="BX6" s="275"/>
-      <c r="BY6" s="275"/>
-      <c r="BZ6" s="275"/>
-      <c r="CA6" s="275"/>
-      <c r="CB6" s="275"/>
+      <c r="BW6" s="267"/>
+      <c r="BX6" s="267"/>
+      <c r="BY6" s="267"/>
+      <c r="BZ6" s="267"/>
+      <c r="CA6" s="267"/>
+      <c r="CB6" s="267"/>
       <c r="CC6" s="71"/>
       <c r="CD6" s="71"/>
     </row>
@@ -7588,356 +7743,356 @@
       <c r="CD7" s="25"/>
     </row>
     <row r="8" spans="1:87" s="11" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A8" s="251" t="s">
+      <c r="A8" s="278" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="279" t="s">
+      <c r="B8" s="271" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="261" t="s">
+      <c r="C8" s="252" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="263" t="s">
+      <c r="D8" s="255" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="263" t="s">
+      <c r="E8" s="255" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="261" t="s">
+      <c r="F8" s="252" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="242" t="s">
+      <c r="G8" s="256" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="270" t="s">
+      <c r="H8" s="262" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="270" t="s">
+      <c r="I8" s="262" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="242" t="s">
+      <c r="J8" s="256" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="271" t="s">
+      <c r="K8" s="276" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="243"/>
-      <c r="M8" s="243"/>
-      <c r="N8" s="243"/>
-      <c r="O8" s="243"/>
-      <c r="P8" s="243"/>
-      <c r="Q8" s="243"/>
-      <c r="R8" s="243"/>
-      <c r="S8" s="243"/>
-      <c r="T8" s="243"/>
-      <c r="U8" s="243"/>
-      <c r="V8" s="243"/>
-      <c r="W8" s="243"/>
-      <c r="X8" s="243"/>
-      <c r="Y8" s="242" t="s">
+      <c r="L8" s="273"/>
+      <c r="M8" s="273"/>
+      <c r="N8" s="273"/>
+      <c r="O8" s="273"/>
+      <c r="P8" s="273"/>
+      <c r="Q8" s="273"/>
+      <c r="R8" s="273"/>
+      <c r="S8" s="273"/>
+      <c r="T8" s="273"/>
+      <c r="U8" s="273"/>
+      <c r="V8" s="273"/>
+      <c r="W8" s="273"/>
+      <c r="X8" s="273"/>
+      <c r="Y8" s="256" t="s">
         <v>15</v>
       </c>
-      <c r="Z8" s="243"/>
-      <c r="AA8" s="243"/>
-      <c r="AB8" s="243"/>
-      <c r="AC8" s="243"/>
-      <c r="AD8" s="243"/>
-      <c r="AE8" s="243"/>
-      <c r="AF8" s="243"/>
-      <c r="AG8" s="243"/>
-      <c r="AH8" s="243"/>
-      <c r="AI8" s="243"/>
-      <c r="AJ8" s="243"/>
-      <c r="AK8" s="243"/>
-      <c r="AL8" s="243"/>
-      <c r="AM8" s="243"/>
-      <c r="AN8" s="243"/>
-      <c r="AO8" s="244"/>
-      <c r="AP8" s="242" t="s">
+      <c r="Z8" s="273"/>
+      <c r="AA8" s="273"/>
+      <c r="AB8" s="273"/>
+      <c r="AC8" s="273"/>
+      <c r="AD8" s="273"/>
+      <c r="AE8" s="273"/>
+      <c r="AF8" s="273"/>
+      <c r="AG8" s="273"/>
+      <c r="AH8" s="273"/>
+      <c r="AI8" s="273"/>
+      <c r="AJ8" s="273"/>
+      <c r="AK8" s="273"/>
+      <c r="AL8" s="273"/>
+      <c r="AM8" s="273"/>
+      <c r="AN8" s="273"/>
+      <c r="AO8" s="274"/>
+      <c r="AP8" s="256" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="242" t="s">
+      <c r="AQ8" s="256" t="s">
         <v>17</v>
       </c>
-      <c r="AR8" s="242" t="s">
+      <c r="AR8" s="256" t="s">
         <v>18</v>
       </c>
-      <c r="AS8" s="242" t="s">
+      <c r="AS8" s="256" t="s">
         <v>19</v>
       </c>
-      <c r="AT8" s="242" t="s">
+      <c r="AT8" s="256" t="s">
         <v>20</v>
       </c>
-      <c r="AU8" s="242" t="s">
+      <c r="AU8" s="256" t="s">
         <v>21</v>
       </c>
-      <c r="AV8" s="261" t="s">
+      <c r="AV8" s="252" t="s">
         <v>22</v>
       </c>
-      <c r="AW8" s="261" t="s">
+      <c r="AW8" s="252" t="s">
         <v>23</v>
       </c>
-      <c r="AX8" s="261" t="s">
+      <c r="AX8" s="252" t="s">
         <v>24</v>
       </c>
-      <c r="AY8" s="268" t="s">
+      <c r="AY8" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ8" s="243"/>
-      <c r="BA8" s="243"/>
-      <c r="BB8" s="243"/>
-      <c r="BC8" s="243"/>
-      <c r="BD8" s="243"/>
-      <c r="BE8" s="243"/>
-      <c r="BF8" s="243"/>
-      <c r="BG8" s="243"/>
-      <c r="BH8" s="243"/>
-      <c r="BI8" s="243"/>
-      <c r="BJ8" s="243"/>
-      <c r="BK8" s="243"/>
-      <c r="BL8" s="243"/>
-      <c r="BM8" s="243"/>
-      <c r="BN8" s="243"/>
-      <c r="BO8" s="243"/>
-      <c r="BP8" s="243"/>
-      <c r="BQ8" s="244"/>
-      <c r="BR8" s="280" t="s">
+      <c r="AZ8" s="273"/>
+      <c r="BA8" s="273"/>
+      <c r="BB8" s="273"/>
+      <c r="BC8" s="273"/>
+      <c r="BD8" s="273"/>
+      <c r="BE8" s="273"/>
+      <c r="BF8" s="273"/>
+      <c r="BG8" s="273"/>
+      <c r="BH8" s="273"/>
+      <c r="BI8" s="273"/>
+      <c r="BJ8" s="273"/>
+      <c r="BK8" s="273"/>
+      <c r="BL8" s="273"/>
+      <c r="BM8" s="273"/>
+      <c r="BN8" s="273"/>
+      <c r="BO8" s="273"/>
+      <c r="BP8" s="273"/>
+      <c r="BQ8" s="274"/>
+      <c r="BR8" s="253" t="s">
         <v>26</v>
       </c>
       <c r="BS8" s="254"/>
-      <c r="BT8" s="268" t="s">
+      <c r="BT8" s="261" t="s">
         <v>27</v>
       </c>
-      <c r="BU8" s="281" t="s">
+      <c r="BU8" s="257" t="s">
         <v>28</v>
       </c>
       <c r="BV8" s="114"/>
-      <c r="BW8" s="262" t="s">
+      <c r="BW8" s="286" t="s">
         <v>29</v>
       </c>
-      <c r="BX8" s="252" t="s">
+      <c r="BX8" s="279" t="s">
         <v>30</v>
       </c>
-      <c r="BY8" s="253"/>
-      <c r="BZ8" s="253"/>
+      <c r="BY8" s="280"/>
+      <c r="BZ8" s="280"/>
       <c r="CA8" s="254"/>
-      <c r="CB8" s="266" t="s">
+      <c r="CB8" s="272" t="s">
         <v>31</v>
       </c>
-      <c r="CC8" s="276" t="s">
+      <c r="CC8" s="244" t="s">
         <v>32</v>
       </c>
-      <c r="CD8" s="276" t="s">
+      <c r="CD8" s="244" t="s">
         <v>33</v>
       </c>
       <c r="CH8" s="27"/>
       <c r="CI8" s="28"/>
     </row>
     <row r="9" spans="1:87" s="11" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A9" s="248"/>
-      <c r="B9" s="248"/>
-      <c r="C9" s="248"/>
-      <c r="D9" s="248"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
-      <c r="G9" s="248"/>
-      <c r="H9" s="248"/>
-      <c r="I9" s="248"/>
-      <c r="J9" s="248"/>
-      <c r="K9" s="247" t="s">
+      <c r="A9" s="245"/>
+      <c r="B9" s="245"/>
+      <c r="C9" s="245"/>
+      <c r="D9" s="245"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="245"/>
+      <c r="G9" s="245"/>
+      <c r="H9" s="245"/>
+      <c r="I9" s="245"/>
+      <c r="J9" s="245"/>
+      <c r="K9" s="258" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="247" t="s">
+      <c r="L9" s="258" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="247" t="s">
+      <c r="M9" s="258" t="s">
         <v>36</v>
       </c>
-      <c r="N9" s="247" t="s">
+      <c r="N9" s="258" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="247" t="s">
+      <c r="O9" s="258" t="s">
         <v>38</v>
       </c>
-      <c r="P9" s="247" t="s">
+      <c r="P9" s="258" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="247" t="s">
+      <c r="Q9" s="258" t="s">
         <v>40</v>
       </c>
-      <c r="R9" s="247" t="s">
+      <c r="R9" s="258" t="s">
         <v>41</v>
       </c>
-      <c r="S9" s="247" t="s">
+      <c r="S9" s="258" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="247" t="s">
+      <c r="T9" s="258" t="s">
         <v>43</v>
       </c>
-      <c r="U9" s="247" t="s">
+      <c r="U9" s="258" t="s">
         <v>44</v>
       </c>
-      <c r="V9" s="284" t="s">
+      <c r="V9" s="263" t="s">
         <v>45</v>
       </c>
       <c r="W9" s="254"/>
-      <c r="X9" s="247" t="s">
+      <c r="X9" s="258" t="s">
         <v>46</v>
       </c>
-      <c r="Y9" s="249" t="s">
+      <c r="Y9" s="247" t="s">
         <v>47</v>
       </c>
-      <c r="Z9" s="249" t="s">
+      <c r="Z9" s="247" t="s">
         <v>48</v>
       </c>
-      <c r="AA9" s="249" t="s">
+      <c r="AA9" s="247" t="s">
         <v>49</v>
       </c>
-      <c r="AB9" s="249" t="s">
+      <c r="AB9" s="247" t="s">
         <v>50</v>
       </c>
-      <c r="AC9" s="250" t="s">
+      <c r="AC9" s="269" t="s">
         <v>51</v>
       </c>
-      <c r="AD9" s="250" t="s">
+      <c r="AD9" s="269" t="s">
         <v>52</v>
       </c>
-      <c r="AE9" s="250" t="s">
+      <c r="AE9" s="269" t="s">
         <v>53</v>
       </c>
-      <c r="AF9" s="250" t="s">
+      <c r="AF9" s="269" t="s">
         <v>54</v>
       </c>
-      <c r="AG9" s="249" t="s">
+      <c r="AG9" s="247" t="s">
         <v>55</v>
       </c>
-      <c r="AH9" s="250" t="s">
+      <c r="AH9" s="269" t="s">
         <v>56</v>
       </c>
-      <c r="AI9" s="250" t="s">
+      <c r="AI9" s="269" t="s">
         <v>57</v>
       </c>
-      <c r="AJ9" s="249" t="s">
+      <c r="AJ9" s="247" t="s">
         <v>58</v>
       </c>
-      <c r="AK9" s="283" t="s">
+      <c r="AK9" s="249" t="s">
         <v>59</v>
       </c>
-      <c r="AL9" s="261" t="s">
+      <c r="AL9" s="252" t="s">
         <v>60</v>
       </c>
-      <c r="AM9" s="249" t="s">
+      <c r="AM9" s="247" t="s">
         <v>61</v>
       </c>
-      <c r="AN9" s="269" t="s">
+      <c r="AN9" s="275" t="s">
         <v>62</v>
       </c>
-      <c r="AO9" s="261" t="s">
+      <c r="AO9" s="252" t="s">
         <v>63</v>
       </c>
-      <c r="AP9" s="248"/>
-      <c r="AQ9" s="248"/>
-      <c r="AR9" s="248"/>
-      <c r="AS9" s="248"/>
-      <c r="AT9" s="248"/>
-      <c r="AU9" s="248"/>
-      <c r="AV9" s="248"/>
-      <c r="AW9" s="248"/>
-      <c r="AX9" s="248"/>
-      <c r="AY9" s="268" t="s">
+      <c r="AP9" s="245"/>
+      <c r="AQ9" s="245"/>
+      <c r="AR9" s="245"/>
+      <c r="AS9" s="245"/>
+      <c r="AT9" s="245"/>
+      <c r="AU9" s="245"/>
+      <c r="AV9" s="245"/>
+      <c r="AW9" s="245"/>
+      <c r="AX9" s="245"/>
+      <c r="AY9" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ9" s="243"/>
-      <c r="BA9" s="243"/>
-      <c r="BB9" s="243"/>
-      <c r="BC9" s="243"/>
-      <c r="BD9" s="243"/>
-      <c r="BE9" s="243"/>
-      <c r="BF9" s="243"/>
-      <c r="BG9" s="243"/>
-      <c r="BH9" s="243"/>
-      <c r="BI9" s="243"/>
-      <c r="BJ9" s="243"/>
-      <c r="BK9" s="243"/>
-      <c r="BL9" s="244"/>
-      <c r="BM9" s="268" t="s">
+      <c r="AZ9" s="273"/>
+      <c r="BA9" s="273"/>
+      <c r="BB9" s="273"/>
+      <c r="BC9" s="273"/>
+      <c r="BD9" s="273"/>
+      <c r="BE9" s="273"/>
+      <c r="BF9" s="273"/>
+      <c r="BG9" s="273"/>
+      <c r="BH9" s="273"/>
+      <c r="BI9" s="273"/>
+      <c r="BJ9" s="273"/>
+      <c r="BK9" s="273"/>
+      <c r="BL9" s="274"/>
+      <c r="BM9" s="261" t="s">
         <v>64</v>
       </c>
-      <c r="BN9" s="243"/>
-      <c r="BO9" s="243"/>
-      <c r="BP9" s="243"/>
-      <c r="BQ9" s="244"/>
-      <c r="BR9" s="265" t="s">
+      <c r="BN9" s="273"/>
+      <c r="BO9" s="273"/>
+      <c r="BP9" s="273"/>
+      <c r="BQ9" s="274"/>
+      <c r="BR9" s="259" t="s">
         <v>65</v>
       </c>
-      <c r="BS9" s="265" t="s">
+      <c r="BS9" s="259" t="s">
         <v>66</v>
       </c>
-      <c r="BT9" s="248"/>
-      <c r="BU9" s="255"/>
+      <c r="BT9" s="245"/>
+      <c r="BU9" s="250"/>
       <c r="BV9" s="114"/>
-      <c r="BW9" s="257"/>
-      <c r="BX9" s="255"/>
-      <c r="BY9" s="256"/>
-      <c r="BZ9" s="256"/>
-      <c r="CA9" s="257"/>
-      <c r="CB9" s="248"/>
-      <c r="CC9" s="248"/>
-      <c r="CD9" s="248"/>
+      <c r="BW9" s="282"/>
+      <c r="BX9" s="250"/>
+      <c r="BY9" s="281"/>
+      <c r="BZ9" s="281"/>
+      <c r="CA9" s="282"/>
+      <c r="CB9" s="245"/>
+      <c r="CC9" s="245"/>
+      <c r="CD9" s="245"/>
       <c r="CH9" s="27"/>
       <c r="CI9" s="28"/>
     </row>
     <row r="10" spans="1:87" s="29" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A10" s="248"/>
-      <c r="B10" s="248"/>
-      <c r="C10" s="248"/>
-      <c r="D10" s="248"/>
-      <c r="E10" s="248"/>
-      <c r="F10" s="248"/>
-      <c r="G10" s="248"/>
-      <c r="H10" s="248"/>
-      <c r="I10" s="248"/>
-      <c r="J10" s="248"/>
-      <c r="K10" s="248"/>
-      <c r="L10" s="248"/>
-      <c r="M10" s="248"/>
-      <c r="N10" s="248"/>
-      <c r="O10" s="248"/>
-      <c r="P10" s="248"/>
-      <c r="Q10" s="248"/>
-      <c r="R10" s="248"/>
-      <c r="S10" s="248"/>
-      <c r="T10" s="248"/>
-      <c r="U10" s="248"/>
-      <c r="V10" s="282"/>
-      <c r="W10" s="285"/>
-      <c r="X10" s="248"/>
-      <c r="Y10" s="248"/>
-      <c r="Z10" s="248"/>
-      <c r="AA10" s="248"/>
-      <c r="AB10" s="248"/>
-      <c r="AC10" s="248"/>
-      <c r="AD10" s="248"/>
-      <c r="AE10" s="248"/>
-      <c r="AF10" s="248"/>
-      <c r="AG10" s="248"/>
-      <c r="AH10" s="248"/>
-      <c r="AI10" s="248"/>
-      <c r="AJ10" s="248"/>
-      <c r="AK10" s="255"/>
-      <c r="AL10" s="248"/>
-      <c r="AM10" s="248"/>
-      <c r="AN10" s="248"/>
-      <c r="AO10" s="248"/>
-      <c r="AP10" s="248"/>
-      <c r="AQ10" s="248"/>
-      <c r="AR10" s="248"/>
-      <c r="AS10" s="248"/>
-      <c r="AT10" s="248"/>
-      <c r="AU10" s="248"/>
-      <c r="AV10" s="248"/>
-      <c r="AW10" s="248"/>
-      <c r="AX10" s="248"/>
+      <c r="A10" s="245"/>
+      <c r="B10" s="245"/>
+      <c r="C10" s="245"/>
+      <c r="D10" s="245"/>
+      <c r="E10" s="245"/>
+      <c r="F10" s="245"/>
+      <c r="G10" s="245"/>
+      <c r="H10" s="245"/>
+      <c r="I10" s="245"/>
+      <c r="J10" s="245"/>
+      <c r="K10" s="245"/>
+      <c r="L10" s="245"/>
+      <c r="M10" s="245"/>
+      <c r="N10" s="245"/>
+      <c r="O10" s="245"/>
+      <c r="P10" s="245"/>
+      <c r="Q10" s="245"/>
+      <c r="R10" s="245"/>
+      <c r="S10" s="245"/>
+      <c r="T10" s="245"/>
+      <c r="U10" s="245"/>
+      <c r="V10" s="251"/>
+      <c r="W10" s="264"/>
+      <c r="X10" s="245"/>
+      <c r="Y10" s="245"/>
+      <c r="Z10" s="245"/>
+      <c r="AA10" s="245"/>
+      <c r="AB10" s="245"/>
+      <c r="AC10" s="245"/>
+      <c r="AD10" s="245"/>
+      <c r="AE10" s="245"/>
+      <c r="AF10" s="245"/>
+      <c r="AG10" s="245"/>
+      <c r="AH10" s="245"/>
+      <c r="AI10" s="245"/>
+      <c r="AJ10" s="245"/>
+      <c r="AK10" s="250"/>
+      <c r="AL10" s="245"/>
+      <c r="AM10" s="245"/>
+      <c r="AN10" s="245"/>
+      <c r="AO10" s="245"/>
+      <c r="AP10" s="245"/>
+      <c r="AQ10" s="245"/>
+      <c r="AR10" s="245"/>
+      <c r="AS10" s="245"/>
+      <c r="AT10" s="245"/>
+      <c r="AU10" s="245"/>
+      <c r="AV10" s="245"/>
+      <c r="AW10" s="245"/>
+      <c r="AX10" s="245"/>
       <c r="AY10" s="101" t="s">
         <v>67</v>
       </c>
@@ -7947,125 +8102,125 @@
       <c r="BA10" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="BB10" s="278" t="s">
+      <c r="BB10" s="270" t="s">
         <v>70</v>
       </c>
-      <c r="BC10" s="245" t="s">
+      <c r="BC10" s="260" t="s">
         <v>71</v>
       </c>
-      <c r="BD10" s="245" t="s">
+      <c r="BD10" s="260" t="s">
         <v>72</v>
       </c>
-      <c r="BE10" s="272" t="s">
+      <c r="BE10" s="277" t="s">
         <v>73</v>
       </c>
-      <c r="BF10" s="245" t="s">
+      <c r="BF10" s="260" t="s">
         <v>74</v>
       </c>
-      <c r="BG10" s="245" t="s">
+      <c r="BG10" s="260" t="s">
         <v>75</v>
       </c>
-      <c r="BH10" s="245" t="s">
+      <c r="BH10" s="260" t="s">
         <v>76</v>
       </c>
-      <c r="BI10" s="245" t="s">
+      <c r="BI10" s="260" t="s">
         <v>77</v>
       </c>
-      <c r="BJ10" s="245" t="s">
+      <c r="BJ10" s="260" t="s">
         <v>78</v>
       </c>
-      <c r="BK10" s="245" t="s">
+      <c r="BK10" s="260" t="s">
         <v>79</v>
       </c>
-      <c r="BL10" s="264" t="s">
+      <c r="BL10" s="287" t="s">
         <v>80</v>
       </c>
-      <c r="BM10" s="245" t="s">
+      <c r="BM10" s="260" t="s">
         <v>81</v>
       </c>
-      <c r="BN10" s="268" t="s">
+      <c r="BN10" s="261" t="s">
         <v>82</v>
       </c>
-      <c r="BO10" s="245" t="s">
+      <c r="BO10" s="260" t="s">
         <v>83</v>
       </c>
-      <c r="BP10" s="268" t="s">
+      <c r="BP10" s="261" t="s">
         <v>84</v>
       </c>
-      <c r="BQ10" s="268" t="s">
+      <c r="BQ10" s="261" t="s">
         <v>85</v>
       </c>
-      <c r="BR10" s="248"/>
-      <c r="BS10" s="248"/>
-      <c r="BT10" s="248"/>
-      <c r="BU10" s="255"/>
+      <c r="BR10" s="245"/>
+      <c r="BS10" s="245"/>
+      <c r="BT10" s="245"/>
+      <c r="BU10" s="250"/>
       <c r="BV10" s="114"/>
-      <c r="BW10" s="257"/>
-      <c r="BX10" s="258"/>
-      <c r="BY10" s="259"/>
-      <c r="BZ10" s="259"/>
-      <c r="CA10" s="260"/>
-      <c r="CB10" s="248"/>
-      <c r="CC10" s="248"/>
-      <c r="CD10" s="248"/>
+      <c r="BW10" s="282"/>
+      <c r="BX10" s="283"/>
+      <c r="BY10" s="284"/>
+      <c r="BZ10" s="284"/>
+      <c r="CA10" s="285"/>
+      <c r="CB10" s="245"/>
+      <c r="CC10" s="245"/>
+      <c r="CD10" s="245"/>
       <c r="CH10" s="27"/>
       <c r="CI10" s="28"/>
     </row>
     <row r="11" spans="1:87" s="29" customFormat="1" ht="38.25" customHeight="1">
-      <c r="A11" s="246"/>
-      <c r="B11" s="246"/>
-      <c r="C11" s="246"/>
-      <c r="D11" s="246"/>
-      <c r="E11" s="246"/>
-      <c r="F11" s="246"/>
-      <c r="G11" s="246"/>
-      <c r="H11" s="246"/>
-      <c r="I11" s="246"/>
-      <c r="J11" s="246"/>
-      <c r="K11" s="246"/>
-      <c r="L11" s="246"/>
-      <c r="M11" s="246"/>
-      <c r="N11" s="246"/>
-      <c r="O11" s="246"/>
-      <c r="P11" s="246"/>
-      <c r="Q11" s="246"/>
-      <c r="R11" s="246"/>
-      <c r="S11" s="246"/>
-      <c r="T11" s="246"/>
-      <c r="U11" s="246"/>
+      <c r="A11" s="248"/>
+      <c r="B11" s="248"/>
+      <c r="C11" s="248"/>
+      <c r="D11" s="248"/>
+      <c r="E11" s="248"/>
+      <c r="F11" s="248"/>
+      <c r="G11" s="248"/>
+      <c r="H11" s="248"/>
+      <c r="I11" s="248"/>
+      <c r="J11" s="248"/>
+      <c r="K11" s="248"/>
+      <c r="L11" s="248"/>
+      <c r="M11" s="248"/>
+      <c r="N11" s="248"/>
+      <c r="O11" s="248"/>
+      <c r="P11" s="248"/>
+      <c r="Q11" s="248"/>
+      <c r="R11" s="248"/>
+      <c r="S11" s="248"/>
+      <c r="T11" s="248"/>
+      <c r="U11" s="248"/>
       <c r="V11" s="30" t="s">
         <v>86</v>
       </c>
       <c r="W11" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="X11" s="246"/>
-      <c r="Y11" s="246"/>
-      <c r="Z11" s="246"/>
-      <c r="AA11" s="246"/>
-      <c r="AB11" s="246"/>
-      <c r="AC11" s="246"/>
-      <c r="AD11" s="246"/>
-      <c r="AE11" s="246"/>
-      <c r="AF11" s="246"/>
-      <c r="AG11" s="246"/>
-      <c r="AH11" s="246"/>
-      <c r="AI11" s="246"/>
-      <c r="AJ11" s="246"/>
-      <c r="AK11" s="282"/>
-      <c r="AL11" s="246"/>
-      <c r="AM11" s="246"/>
-      <c r="AN11" s="246"/>
-      <c r="AO11" s="246"/>
-      <c r="AP11" s="246"/>
-      <c r="AQ11" s="246"/>
-      <c r="AR11" s="246"/>
-      <c r="AS11" s="246"/>
-      <c r="AT11" s="246"/>
-      <c r="AU11" s="246"/>
-      <c r="AV11" s="246"/>
-      <c r="AW11" s="246"/>
-      <c r="AX11" s="246"/>
+      <c r="X11" s="248"/>
+      <c r="Y11" s="248"/>
+      <c r="Z11" s="248"/>
+      <c r="AA11" s="248"/>
+      <c r="AB11" s="248"/>
+      <c r="AC11" s="248"/>
+      <c r="AD11" s="248"/>
+      <c r="AE11" s="248"/>
+      <c r="AF11" s="248"/>
+      <c r="AG11" s="248"/>
+      <c r="AH11" s="248"/>
+      <c r="AI11" s="248"/>
+      <c r="AJ11" s="248"/>
+      <c r="AK11" s="251"/>
+      <c r="AL11" s="248"/>
+      <c r="AM11" s="248"/>
+      <c r="AN11" s="248"/>
+      <c r="AO11" s="248"/>
+      <c r="AP11" s="248"/>
+      <c r="AQ11" s="248"/>
+      <c r="AR11" s="248"/>
+      <c r="AS11" s="248"/>
+      <c r="AT11" s="248"/>
+      <c r="AU11" s="248"/>
+      <c r="AV11" s="248"/>
+      <c r="AW11" s="248"/>
+      <c r="AX11" s="248"/>
       <c r="AY11" s="102" t="s">
         <v>88</v>
       </c>
@@ -8075,28 +8230,28 @@
       <c r="BA11" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="BB11" s="246"/>
-      <c r="BC11" s="246"/>
-      <c r="BD11" s="246"/>
-      <c r="BE11" s="246"/>
-      <c r="BF11" s="246"/>
-      <c r="BG11" s="246"/>
-      <c r="BH11" s="246"/>
-      <c r="BI11" s="246"/>
-      <c r="BJ11" s="246"/>
-      <c r="BK11" s="246"/>
-      <c r="BL11" s="246"/>
-      <c r="BM11" s="246"/>
-      <c r="BN11" s="246"/>
-      <c r="BO11" s="246"/>
-      <c r="BP11" s="246"/>
-      <c r="BQ11" s="246"/>
-      <c r="BR11" s="246"/>
-      <c r="BS11" s="246"/>
-      <c r="BT11" s="246"/>
-      <c r="BU11" s="282"/>
+      <c r="BB11" s="248"/>
+      <c r="BC11" s="248"/>
+      <c r="BD11" s="248"/>
+      <c r="BE11" s="248"/>
+      <c r="BF11" s="248"/>
+      <c r="BG11" s="248"/>
+      <c r="BH11" s="248"/>
+      <c r="BI11" s="248"/>
+      <c r="BJ11" s="248"/>
+      <c r="BK11" s="248"/>
+      <c r="BL11" s="248"/>
+      <c r="BM11" s="248"/>
+      <c r="BN11" s="248"/>
+      <c r="BO11" s="248"/>
+      <c r="BP11" s="248"/>
+      <c r="BQ11" s="248"/>
+      <c r="BR11" s="248"/>
+      <c r="BS11" s="248"/>
+      <c r="BT11" s="248"/>
+      <c r="BU11" s="251"/>
       <c r="BV11" s="114"/>
-      <c r="BW11" s="260"/>
+      <c r="BW11" s="285"/>
       <c r="BX11" s="72" t="s">
         <v>91</v>
       </c>
@@ -8109,9 +8264,9 @@
       <c r="CA11" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="CB11" s="267"/>
-      <c r="CC11" s="267"/>
-      <c r="CD11" s="267"/>
+      <c r="CB11" s="246"/>
+      <c r="CC11" s="246"/>
+      <c r="CD11" s="246"/>
       <c r="CE11" s="11"/>
       <c r="CF11" s="31"/>
       <c r="CH11" s="27"/>
@@ -10636,34 +10791,47 @@
       <c r="CF24" s="57"/>
     </row>
     <row r="27" spans="1:87" ht="17">
-      <c r="B27" s="299" t="s">
+      <c r="B27" s="242" t="s">
         <v>150</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A12:CI21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="82">
-    <mergeCell ref="CD8:CD11"/>
-    <mergeCell ref="Y9:Y11"/>
-    <mergeCell ref="AA9:AA11"/>
-    <mergeCell ref="AK9:AK11"/>
-    <mergeCell ref="AM9:AM11"/>
-    <mergeCell ref="AX8:AX11"/>
-    <mergeCell ref="BR8:BS8"/>
-    <mergeCell ref="E8:E11"/>
-    <mergeCell ref="G8:G11"/>
-    <mergeCell ref="BU8:BU11"/>
-    <mergeCell ref="R9:R11"/>
-    <mergeCell ref="BR9:BR11"/>
-    <mergeCell ref="BM10:BM11"/>
-    <mergeCell ref="AQ8:AQ11"/>
-    <mergeCell ref="U9:U11"/>
-    <mergeCell ref="BN10:BN11"/>
-    <mergeCell ref="BP10:BP11"/>
-    <mergeCell ref="AG9:AG11"/>
-    <mergeCell ref="H8:H11"/>
-    <mergeCell ref="J8:J11"/>
-    <mergeCell ref="V9:W10"/>
+    <mergeCell ref="AF9:AF11"/>
+    <mergeCell ref="AH9:AH11"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="BX8:CA10"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="BW8:BW11"/>
+    <mergeCell ref="AI9:AI11"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="BF10:BF11"/>
+    <mergeCell ref="BO10:BO11"/>
+    <mergeCell ref="Q9:Q11"/>
+    <mergeCell ref="S9:S11"/>
+    <mergeCell ref="BL10:BL11"/>
+    <mergeCell ref="BS9:BS11"/>
+    <mergeCell ref="AC9:AC11"/>
+    <mergeCell ref="AP8:AP11"/>
+    <mergeCell ref="AR8:AR11"/>
+    <mergeCell ref="AT8:AT11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="BK10:BK11"/>
+    <mergeCell ref="K8:X8"/>
+    <mergeCell ref="AY8:BQ8"/>
+    <mergeCell ref="BC10:BC11"/>
+    <mergeCell ref="BE10:BE11"/>
+    <mergeCell ref="T9:T11"/>
+    <mergeCell ref="BQ10:BQ11"/>
+    <mergeCell ref="AB9:AB11"/>
+    <mergeCell ref="Y8:AO8"/>
+    <mergeCell ref="BJ10:BJ11"/>
+    <mergeCell ref="L9:L11"/>
+    <mergeCell ref="N9:N11"/>
+    <mergeCell ref="BG10:BG11"/>
+    <mergeCell ref="BI10:BI11"/>
+    <mergeCell ref="X9:X11"/>
     <mergeCell ref="BW3:CB6"/>
     <mergeCell ref="CC8:CC11"/>
     <mergeCell ref="AU8:AU11"/>
@@ -10680,51 +10848,38 @@
     <mergeCell ref="BH10:BH11"/>
     <mergeCell ref="BT8:BT11"/>
     <mergeCell ref="P9:P11"/>
+    <mergeCell ref="E8:E11"/>
+    <mergeCell ref="G8:G11"/>
+    <mergeCell ref="BU8:BU11"/>
+    <mergeCell ref="R9:R11"/>
+    <mergeCell ref="BR9:BR11"/>
+    <mergeCell ref="BM10:BM11"/>
+    <mergeCell ref="AQ8:AQ11"/>
+    <mergeCell ref="U9:U11"/>
+    <mergeCell ref="BN10:BN11"/>
+    <mergeCell ref="BP10:BP11"/>
+    <mergeCell ref="AG9:AG11"/>
+    <mergeCell ref="H8:H11"/>
+    <mergeCell ref="J8:J11"/>
+    <mergeCell ref="V9:W10"/>
     <mergeCell ref="F8:F11"/>
+    <mergeCell ref="AJ9:AJ11"/>
+    <mergeCell ref="CD8:CD11"/>
+    <mergeCell ref="Y9:Y11"/>
+    <mergeCell ref="AA9:AA11"/>
+    <mergeCell ref="AK9:AK11"/>
+    <mergeCell ref="AM9:AM11"/>
+    <mergeCell ref="AX8:AX11"/>
+    <mergeCell ref="BR8:BS8"/>
     <mergeCell ref="CB8:CB11"/>
-    <mergeCell ref="AJ9:AJ11"/>
     <mergeCell ref="AL9:AL11"/>
     <mergeCell ref="AY9:BL9"/>
     <mergeCell ref="AN9:AN11"/>
     <mergeCell ref="BM9:BQ9"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="BK10:BK11"/>
-    <mergeCell ref="K8:X8"/>
-    <mergeCell ref="AY8:BQ8"/>
-    <mergeCell ref="BC10:BC11"/>
-    <mergeCell ref="BE10:BE11"/>
-    <mergeCell ref="T9:T11"/>
-    <mergeCell ref="BQ10:BQ11"/>
-    <mergeCell ref="AB9:AB11"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="BX8:CA10"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="BW8:BW11"/>
-    <mergeCell ref="AI9:AI11"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="BF10:BF11"/>
-    <mergeCell ref="BO10:BO11"/>
-    <mergeCell ref="Q9:Q11"/>
-    <mergeCell ref="S9:S11"/>
-    <mergeCell ref="BL10:BL11"/>
-    <mergeCell ref="BS9:BS11"/>
-    <mergeCell ref="AC9:AC11"/>
-    <mergeCell ref="AP8:AP11"/>
-    <mergeCell ref="AR8:AR11"/>
-    <mergeCell ref="AT8:AT11"/>
-    <mergeCell ref="Y8:AO8"/>
-    <mergeCell ref="BJ10:BJ11"/>
-    <mergeCell ref="L9:L11"/>
-    <mergeCell ref="N9:N11"/>
-    <mergeCell ref="BG10:BG11"/>
-    <mergeCell ref="BI10:BI11"/>
-    <mergeCell ref="X9:X11"/>
     <mergeCell ref="Z9:Z11"/>
     <mergeCell ref="AD9:AD11"/>
     <mergeCell ref="AS8:AS11"/>
     <mergeCell ref="AV8:AV11"/>
-    <mergeCell ref="AF9:AF11"/>
-    <mergeCell ref="AH9:AH11"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B12 B15:B26 C12:BU12 B28:B1048576">
     <cfRule type="duplicateValues" dxfId="23" priority="36"/>
@@ -10933,7 +11088,7 @@
       <c r="CD2" s="137"/>
     </row>
     <row r="3" spans="1:87" s="139" customFormat="1" ht="11" outlineLevel="1">
-      <c r="A3" s="290"/>
+      <c r="A3" s="293"/>
       <c r="B3" s="291"/>
       <c r="C3" s="291"/>
       <c r="D3" s="291"/>
@@ -11006,7 +11161,7 @@
       <c r="BS3" s="291"/>
       <c r="BT3" s="291"/>
       <c r="BU3" s="291"/>
-      <c r="BW3" s="293" t="s">
+      <c r="BW3" s="290" t="s">
         <v>2</v>
       </c>
       <c r="BX3" s="291"/>
@@ -11106,354 +11261,354 @@
       <c r="CD4" s="138"/>
     </row>
     <row r="5" spans="1:87" s="141" customFormat="1">
-      <c r="A5" s="251" t="s">
+      <c r="A5" s="278" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="279" t="s">
+      <c r="B5" s="271" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="261" t="s">
+      <c r="C5" s="252" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="263" t="s">
+      <c r="D5" s="255" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="263" t="s">
+      <c r="E5" s="255" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="261" t="s">
+      <c r="F5" s="252" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="261" t="s">
+      <c r="G5" s="252" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="287" t="s">
+      <c r="H5" s="289" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="287" t="s">
+      <c r="I5" s="289" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="261" t="s">
+      <c r="J5" s="252" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="288" t="s">
+      <c r="K5" s="294" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="243"/>
-      <c r="M5" s="243"/>
-      <c r="N5" s="243"/>
-      <c r="O5" s="243"/>
-      <c r="P5" s="243"/>
-      <c r="Q5" s="243"/>
-      <c r="R5" s="243"/>
-      <c r="S5" s="243"/>
-      <c r="T5" s="243"/>
-      <c r="U5" s="243"/>
-      <c r="V5" s="243"/>
-      <c r="W5" s="243"/>
-      <c r="X5" s="243"/>
-      <c r="Y5" s="261" t="s">
+      <c r="L5" s="273"/>
+      <c r="M5" s="273"/>
+      <c r="N5" s="273"/>
+      <c r="O5" s="273"/>
+      <c r="P5" s="273"/>
+      <c r="Q5" s="273"/>
+      <c r="R5" s="273"/>
+      <c r="S5" s="273"/>
+      <c r="T5" s="273"/>
+      <c r="U5" s="273"/>
+      <c r="V5" s="273"/>
+      <c r="W5" s="273"/>
+      <c r="X5" s="273"/>
+      <c r="Y5" s="252" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="243"/>
-      <c r="AA5" s="243"/>
-      <c r="AB5" s="243"/>
-      <c r="AC5" s="243"/>
-      <c r="AD5" s="243"/>
-      <c r="AE5" s="243"/>
-      <c r="AF5" s="243"/>
-      <c r="AG5" s="243"/>
-      <c r="AH5" s="243"/>
-      <c r="AI5" s="243"/>
-      <c r="AJ5" s="243"/>
-      <c r="AK5" s="243"/>
-      <c r="AL5" s="243"/>
-      <c r="AM5" s="243"/>
-      <c r="AN5" s="243"/>
-      <c r="AO5" s="244"/>
-      <c r="AP5" s="261" t="s">
+      <c r="Z5" s="273"/>
+      <c r="AA5" s="273"/>
+      <c r="AB5" s="273"/>
+      <c r="AC5" s="273"/>
+      <c r="AD5" s="273"/>
+      <c r="AE5" s="273"/>
+      <c r="AF5" s="273"/>
+      <c r="AG5" s="273"/>
+      <c r="AH5" s="273"/>
+      <c r="AI5" s="273"/>
+      <c r="AJ5" s="273"/>
+      <c r="AK5" s="273"/>
+      <c r="AL5" s="273"/>
+      <c r="AM5" s="273"/>
+      <c r="AN5" s="273"/>
+      <c r="AO5" s="274"/>
+      <c r="AP5" s="252" t="s">
         <v>16</v>
       </c>
-      <c r="AQ5" s="261" t="s">
+      <c r="AQ5" s="252" t="s">
         <v>17</v>
       </c>
-      <c r="AR5" s="261" t="s">
+      <c r="AR5" s="252" t="s">
         <v>18</v>
       </c>
-      <c r="AS5" s="261" t="s">
+      <c r="AS5" s="252" t="s">
         <v>19</v>
       </c>
-      <c r="AT5" s="261" t="s">
+      <c r="AT5" s="252" t="s">
         <v>20</v>
       </c>
-      <c r="AU5" s="261" t="s">
+      <c r="AU5" s="252" t="s">
         <v>21</v>
       </c>
-      <c r="AV5" s="261" t="s">
+      <c r="AV5" s="252" t="s">
         <v>22</v>
       </c>
-      <c r="AW5" s="261" t="s">
+      <c r="AW5" s="252" t="s">
         <v>23</v>
       </c>
-      <c r="AX5" s="261" t="s">
+      <c r="AX5" s="252" t="s">
         <v>24</v>
       </c>
-      <c r="AY5" s="268" t="s">
+      <c r="AY5" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ5" s="243"/>
-      <c r="BA5" s="243"/>
-      <c r="BB5" s="243"/>
-      <c r="BC5" s="243"/>
-      <c r="BD5" s="243"/>
-      <c r="BE5" s="243"/>
-      <c r="BF5" s="243"/>
-      <c r="BG5" s="243"/>
-      <c r="BH5" s="243"/>
-      <c r="BI5" s="243"/>
-      <c r="BJ5" s="243"/>
-      <c r="BK5" s="243"/>
-      <c r="BL5" s="243"/>
-      <c r="BM5" s="243"/>
-      <c r="BN5" s="243"/>
-      <c r="BO5" s="243"/>
-      <c r="BP5" s="243"/>
-      <c r="BQ5" s="244"/>
-      <c r="BR5" s="280" t="s">
+      <c r="AZ5" s="273"/>
+      <c r="BA5" s="273"/>
+      <c r="BB5" s="273"/>
+      <c r="BC5" s="273"/>
+      <c r="BD5" s="273"/>
+      <c r="BE5" s="273"/>
+      <c r="BF5" s="273"/>
+      <c r="BG5" s="273"/>
+      <c r="BH5" s="273"/>
+      <c r="BI5" s="273"/>
+      <c r="BJ5" s="273"/>
+      <c r="BK5" s="273"/>
+      <c r="BL5" s="273"/>
+      <c r="BM5" s="273"/>
+      <c r="BN5" s="273"/>
+      <c r="BO5" s="273"/>
+      <c r="BP5" s="273"/>
+      <c r="BQ5" s="274"/>
+      <c r="BR5" s="253" t="s">
         <v>26</v>
       </c>
       <c r="BS5" s="254"/>
-      <c r="BT5" s="268" t="s">
+      <c r="BT5" s="261" t="s">
         <v>27</v>
       </c>
-      <c r="BU5" s="281" t="s">
+      <c r="BU5" s="257" t="s">
         <v>28</v>
       </c>
-      <c r="BW5" s="262" t="s">
+      <c r="BW5" s="286" t="s">
         <v>29</v>
       </c>
-      <c r="BX5" s="252" t="s">
+      <c r="BX5" s="279" t="s">
         <v>30</v>
       </c>
-      <c r="BY5" s="253"/>
-      <c r="BZ5" s="253"/>
+      <c r="BY5" s="280"/>
+      <c r="BZ5" s="280"/>
       <c r="CA5" s="254"/>
-      <c r="CB5" s="266" t="s">
+      <c r="CB5" s="272" t="s">
         <v>31</v>
       </c>
-      <c r="CC5" s="276" t="s">
+      <c r="CC5" s="244" t="s">
         <v>32</v>
       </c>
-      <c r="CD5" s="276" t="s">
+      <c r="CD5" s="244" t="s">
         <v>33</v>
       </c>
       <c r="CH5" s="142"/>
       <c r="CI5" s="143"/>
     </row>
     <row r="6" spans="1:87" s="141" customFormat="1">
-      <c r="A6" s="248"/>
-      <c r="B6" s="248"/>
-      <c r="C6" s="248"/>
-      <c r="D6" s="248"/>
-      <c r="E6" s="248"/>
-      <c r="F6" s="248"/>
-      <c r="G6" s="248"/>
-      <c r="H6" s="248"/>
-      <c r="I6" s="248"/>
-      <c r="J6" s="248"/>
-      <c r="K6" s="286" t="s">
+      <c r="A6" s="245"/>
+      <c r="B6" s="245"/>
+      <c r="C6" s="245"/>
+      <c r="D6" s="245"/>
+      <c r="E6" s="245"/>
+      <c r="F6" s="245"/>
+      <c r="G6" s="245"/>
+      <c r="H6" s="245"/>
+      <c r="I6" s="245"/>
+      <c r="J6" s="245"/>
+      <c r="K6" s="288" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="286" t="s">
+      <c r="L6" s="288" t="s">
         <v>35</v>
       </c>
-      <c r="M6" s="286" t="s">
+      <c r="M6" s="288" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="286" t="s">
+      <c r="N6" s="288" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="286" t="s">
+      <c r="O6" s="288" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="286" t="s">
+      <c r="P6" s="288" t="s">
         <v>39</v>
       </c>
-      <c r="Q6" s="286" t="s">
+      <c r="Q6" s="288" t="s">
         <v>40</v>
       </c>
-      <c r="R6" s="286" t="s">
+      <c r="R6" s="288" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="286" t="s">
+      <c r="S6" s="288" t="s">
         <v>42</v>
       </c>
-      <c r="T6" s="286" t="s">
+      <c r="T6" s="288" t="s">
         <v>43</v>
       </c>
-      <c r="U6" s="286" t="s">
+      <c r="U6" s="288" t="s">
         <v>44</v>
       </c>
-      <c r="V6" s="289" t="s">
+      <c r="V6" s="295" t="s">
         <v>45</v>
       </c>
       <c r="W6" s="254"/>
-      <c r="X6" s="286" t="s">
+      <c r="X6" s="288" t="s">
         <v>46</v>
       </c>
-      <c r="Y6" s="261" t="s">
+      <c r="Y6" s="252" t="s">
         <v>47</v>
       </c>
-      <c r="Z6" s="261" t="s">
+      <c r="Z6" s="252" t="s">
         <v>48</v>
       </c>
-      <c r="AA6" s="261" t="s">
+      <c r="AA6" s="252" t="s">
         <v>49</v>
       </c>
-      <c r="AB6" s="261" t="s">
+      <c r="AB6" s="252" t="s">
         <v>50</v>
       </c>
-      <c r="AC6" s="287" t="s">
+      <c r="AC6" s="289" t="s">
         <v>51</v>
       </c>
-      <c r="AD6" s="287" t="s">
+      <c r="AD6" s="289" t="s">
         <v>52</v>
       </c>
-      <c r="AE6" s="287" t="s">
+      <c r="AE6" s="289" t="s">
         <v>53</v>
       </c>
-      <c r="AF6" s="287" t="s">
+      <c r="AF6" s="289" t="s">
         <v>54</v>
       </c>
-      <c r="AG6" s="261" t="s">
+      <c r="AG6" s="252" t="s">
         <v>55</v>
       </c>
-      <c r="AH6" s="287" t="s">
+      <c r="AH6" s="289" t="s">
         <v>56</v>
       </c>
-      <c r="AI6" s="287" t="s">
+      <c r="AI6" s="289" t="s">
         <v>57</v>
       </c>
-      <c r="AJ6" s="261" t="s">
+      <c r="AJ6" s="252" t="s">
         <v>58</v>
       </c>
-      <c r="AK6" s="283" t="s">
+      <c r="AK6" s="249" t="s">
         <v>59</v>
       </c>
-      <c r="AL6" s="261" t="s">
+      <c r="AL6" s="252" t="s">
         <v>60</v>
       </c>
-      <c r="AM6" s="261" t="s">
+      <c r="AM6" s="252" t="s">
         <v>61</v>
       </c>
-      <c r="AN6" s="269" t="s">
+      <c r="AN6" s="275" t="s">
         <v>62</v>
       </c>
-      <c r="AO6" s="261" t="s">
+      <c r="AO6" s="252" t="s">
         <v>63</v>
       </c>
-      <c r="AP6" s="248"/>
-      <c r="AQ6" s="248"/>
-      <c r="AR6" s="248"/>
-      <c r="AS6" s="248"/>
-      <c r="AT6" s="248"/>
-      <c r="AU6" s="248"/>
-      <c r="AV6" s="248"/>
-      <c r="AW6" s="248"/>
-      <c r="AX6" s="248"/>
-      <c r="AY6" s="268" t="s">
+      <c r="AP6" s="245"/>
+      <c r="AQ6" s="245"/>
+      <c r="AR6" s="245"/>
+      <c r="AS6" s="245"/>
+      <c r="AT6" s="245"/>
+      <c r="AU6" s="245"/>
+      <c r="AV6" s="245"/>
+      <c r="AW6" s="245"/>
+      <c r="AX6" s="245"/>
+      <c r="AY6" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ6" s="243"/>
-      <c r="BA6" s="243"/>
-      <c r="BB6" s="243"/>
-      <c r="BC6" s="243"/>
-      <c r="BD6" s="243"/>
-      <c r="BE6" s="243"/>
-      <c r="BF6" s="243"/>
-      <c r="BG6" s="243"/>
-      <c r="BH6" s="243"/>
-      <c r="BI6" s="243"/>
-      <c r="BJ6" s="243"/>
-      <c r="BK6" s="243"/>
-      <c r="BL6" s="244"/>
-      <c r="BM6" s="268" t="s">
+      <c r="AZ6" s="273"/>
+      <c r="BA6" s="273"/>
+      <c r="BB6" s="273"/>
+      <c r="BC6" s="273"/>
+      <c r="BD6" s="273"/>
+      <c r="BE6" s="273"/>
+      <c r="BF6" s="273"/>
+      <c r="BG6" s="273"/>
+      <c r="BH6" s="273"/>
+      <c r="BI6" s="273"/>
+      <c r="BJ6" s="273"/>
+      <c r="BK6" s="273"/>
+      <c r="BL6" s="274"/>
+      <c r="BM6" s="261" t="s">
         <v>64</v>
       </c>
-      <c r="BN6" s="243"/>
-      <c r="BO6" s="243"/>
-      <c r="BP6" s="243"/>
-      <c r="BQ6" s="244"/>
-      <c r="BR6" s="265" t="s">
+      <c r="BN6" s="273"/>
+      <c r="BO6" s="273"/>
+      <c r="BP6" s="273"/>
+      <c r="BQ6" s="274"/>
+      <c r="BR6" s="259" t="s">
         <v>65</v>
       </c>
-      <c r="BS6" s="265" t="s">
+      <c r="BS6" s="259" t="s">
         <v>66</v>
       </c>
-      <c r="BT6" s="248"/>
-      <c r="BU6" s="255"/>
-      <c r="BW6" s="257"/>
-      <c r="BX6" s="255"/>
+      <c r="BT6" s="245"/>
+      <c r="BU6" s="250"/>
+      <c r="BW6" s="282"/>
+      <c r="BX6" s="250"/>
       <c r="BY6" s="292"/>
       <c r="BZ6" s="292"/>
-      <c r="CA6" s="257"/>
-      <c r="CB6" s="248"/>
-      <c r="CC6" s="248"/>
-      <c r="CD6" s="248"/>
+      <c r="CA6" s="282"/>
+      <c r="CB6" s="245"/>
+      <c r="CC6" s="245"/>
+      <c r="CD6" s="245"/>
       <c r="CH6" s="142"/>
       <c r="CI6" s="143"/>
     </row>
     <row r="7" spans="1:87" s="144" customFormat="1" ht="12">
-      <c r="A7" s="248"/>
-      <c r="B7" s="248"/>
-      <c r="C7" s="248"/>
-      <c r="D7" s="248"/>
-      <c r="E7" s="248"/>
-      <c r="F7" s="248"/>
-      <c r="G7" s="248"/>
-      <c r="H7" s="248"/>
-      <c r="I7" s="248"/>
-      <c r="J7" s="248"/>
-      <c r="K7" s="248"/>
-      <c r="L7" s="248"/>
-      <c r="M7" s="248"/>
-      <c r="N7" s="248"/>
-      <c r="O7" s="248"/>
-      <c r="P7" s="248"/>
-      <c r="Q7" s="248"/>
-      <c r="R7" s="248"/>
-      <c r="S7" s="248"/>
-      <c r="T7" s="248"/>
-      <c r="U7" s="248"/>
-      <c r="V7" s="282"/>
-      <c r="W7" s="285"/>
-      <c r="X7" s="248"/>
-      <c r="Y7" s="248"/>
-      <c r="Z7" s="248"/>
-      <c r="AA7" s="248"/>
-      <c r="AB7" s="248"/>
-      <c r="AC7" s="248"/>
-      <c r="AD7" s="248"/>
-      <c r="AE7" s="248"/>
-      <c r="AF7" s="248"/>
-      <c r="AG7" s="248"/>
-      <c r="AH7" s="248"/>
-      <c r="AI7" s="248"/>
-      <c r="AJ7" s="248"/>
-      <c r="AK7" s="255"/>
-      <c r="AL7" s="248"/>
-      <c r="AM7" s="248"/>
-      <c r="AN7" s="248"/>
-      <c r="AO7" s="248"/>
-      <c r="AP7" s="248"/>
-      <c r="AQ7" s="248"/>
-      <c r="AR7" s="248"/>
-      <c r="AS7" s="248"/>
-      <c r="AT7" s="248"/>
-      <c r="AU7" s="248"/>
-      <c r="AV7" s="248"/>
-      <c r="AW7" s="248"/>
-      <c r="AX7" s="248"/>
+      <c r="A7" s="245"/>
+      <c r="B7" s="245"/>
+      <c r="C7" s="245"/>
+      <c r="D7" s="245"/>
+      <c r="E7" s="245"/>
+      <c r="F7" s="245"/>
+      <c r="G7" s="245"/>
+      <c r="H7" s="245"/>
+      <c r="I7" s="245"/>
+      <c r="J7" s="245"/>
+      <c r="K7" s="245"/>
+      <c r="L7" s="245"/>
+      <c r="M7" s="245"/>
+      <c r="N7" s="245"/>
+      <c r="O7" s="245"/>
+      <c r="P7" s="245"/>
+      <c r="Q7" s="245"/>
+      <c r="R7" s="245"/>
+      <c r="S7" s="245"/>
+      <c r="T7" s="245"/>
+      <c r="U7" s="245"/>
+      <c r="V7" s="251"/>
+      <c r="W7" s="264"/>
+      <c r="X7" s="245"/>
+      <c r="Y7" s="245"/>
+      <c r="Z7" s="245"/>
+      <c r="AA7" s="245"/>
+      <c r="AB7" s="245"/>
+      <c r="AC7" s="245"/>
+      <c r="AD7" s="245"/>
+      <c r="AE7" s="245"/>
+      <c r="AF7" s="245"/>
+      <c r="AG7" s="245"/>
+      <c r="AH7" s="245"/>
+      <c r="AI7" s="245"/>
+      <c r="AJ7" s="245"/>
+      <c r="AK7" s="250"/>
+      <c r="AL7" s="245"/>
+      <c r="AM7" s="245"/>
+      <c r="AN7" s="245"/>
+      <c r="AO7" s="245"/>
+      <c r="AP7" s="245"/>
+      <c r="AQ7" s="245"/>
+      <c r="AR7" s="245"/>
+      <c r="AS7" s="245"/>
+      <c r="AT7" s="245"/>
+      <c r="AU7" s="245"/>
+      <c r="AV7" s="245"/>
+      <c r="AW7" s="245"/>
+      <c r="AX7" s="245"/>
       <c r="AY7" s="101" t="s">
         <v>67</v>
       </c>
@@ -11463,124 +11618,124 @@
       <c r="BA7" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="BB7" s="268" t="s">
+      <c r="BB7" s="261" t="s">
         <v>70</v>
       </c>
-      <c r="BC7" s="245" t="s">
+      <c r="BC7" s="260" t="s">
         <v>71</v>
       </c>
-      <c r="BD7" s="245" t="s">
+      <c r="BD7" s="260" t="s">
         <v>72</v>
       </c>
-      <c r="BE7" s="272" t="s">
+      <c r="BE7" s="277" t="s">
         <v>73</v>
       </c>
-      <c r="BF7" s="245" t="s">
+      <c r="BF7" s="260" t="s">
         <v>74</v>
       </c>
-      <c r="BG7" s="245" t="s">
+      <c r="BG7" s="260" t="s">
         <v>75</v>
       </c>
-      <c r="BH7" s="245" t="s">
+      <c r="BH7" s="260" t="s">
         <v>76</v>
       </c>
-      <c r="BI7" s="245" t="s">
+      <c r="BI7" s="260" t="s">
         <v>77</v>
       </c>
-      <c r="BJ7" s="245" t="s">
+      <c r="BJ7" s="260" t="s">
         <v>78</v>
       </c>
-      <c r="BK7" s="245" t="s">
+      <c r="BK7" s="260" t="s">
         <v>79</v>
       </c>
-      <c r="BL7" s="264" t="s">
+      <c r="BL7" s="287" t="s">
         <v>80</v>
       </c>
-      <c r="BM7" s="245" t="s">
+      <c r="BM7" s="260" t="s">
         <v>81</v>
       </c>
-      <c r="BN7" s="268" t="s">
+      <c r="BN7" s="261" t="s">
         <v>82</v>
       </c>
-      <c r="BO7" s="245" t="s">
+      <c r="BO7" s="260" t="s">
         <v>83</v>
       </c>
-      <c r="BP7" s="268" t="s">
+      <c r="BP7" s="261" t="s">
         <v>84</v>
       </c>
-      <c r="BQ7" s="268" t="s">
+      <c r="BQ7" s="261" t="s">
         <v>85</v>
       </c>
-      <c r="BR7" s="248"/>
-      <c r="BS7" s="248"/>
-      <c r="BT7" s="248"/>
-      <c r="BU7" s="255"/>
-      <c r="BW7" s="257"/>
-      <c r="BX7" s="258"/>
-      <c r="BY7" s="259"/>
-      <c r="BZ7" s="259"/>
-      <c r="CA7" s="260"/>
-      <c r="CB7" s="248"/>
-      <c r="CC7" s="248"/>
-      <c r="CD7" s="248"/>
+      <c r="BR7" s="245"/>
+      <c r="BS7" s="245"/>
+      <c r="BT7" s="245"/>
+      <c r="BU7" s="250"/>
+      <c r="BW7" s="282"/>
+      <c r="BX7" s="283"/>
+      <c r="BY7" s="284"/>
+      <c r="BZ7" s="284"/>
+      <c r="CA7" s="285"/>
+      <c r="CB7" s="245"/>
+      <c r="CC7" s="245"/>
+      <c r="CD7" s="245"/>
       <c r="CH7" s="142"/>
       <c r="CI7" s="143"/>
     </row>
     <row r="8" spans="1:87" s="144" customFormat="1" ht="12">
-      <c r="A8" s="246"/>
-      <c r="B8" s="246"/>
-      <c r="C8" s="246"/>
-      <c r="D8" s="246"/>
-      <c r="E8" s="246"/>
-      <c r="F8" s="246"/>
-      <c r="G8" s="246"/>
-      <c r="H8" s="246"/>
-      <c r="I8" s="246"/>
-      <c r="J8" s="246"/>
-      <c r="K8" s="246"/>
-      <c r="L8" s="246"/>
-      <c r="M8" s="246"/>
-      <c r="N8" s="246"/>
-      <c r="O8" s="246"/>
-      <c r="P8" s="246"/>
-      <c r="Q8" s="246"/>
-      <c r="R8" s="246"/>
-      <c r="S8" s="246"/>
-      <c r="T8" s="246"/>
-      <c r="U8" s="246"/>
+      <c r="A8" s="248"/>
+      <c r="B8" s="248"/>
+      <c r="C8" s="248"/>
+      <c r="D8" s="248"/>
+      <c r="E8" s="248"/>
+      <c r="F8" s="248"/>
+      <c r="G8" s="248"/>
+      <c r="H8" s="248"/>
+      <c r="I8" s="248"/>
+      <c r="J8" s="248"/>
+      <c r="K8" s="248"/>
+      <c r="L8" s="248"/>
+      <c r="M8" s="248"/>
+      <c r="N8" s="248"/>
+      <c r="O8" s="248"/>
+      <c r="P8" s="248"/>
+      <c r="Q8" s="248"/>
+      <c r="R8" s="248"/>
+      <c r="S8" s="248"/>
+      <c r="T8" s="248"/>
+      <c r="U8" s="248"/>
       <c r="V8" s="145" t="s">
         <v>86</v>
       </c>
       <c r="W8" s="145" t="s">
         <v>87</v>
       </c>
-      <c r="X8" s="246"/>
-      <c r="Y8" s="246"/>
-      <c r="Z8" s="246"/>
-      <c r="AA8" s="246"/>
-      <c r="AB8" s="246"/>
-      <c r="AC8" s="246"/>
-      <c r="AD8" s="246"/>
-      <c r="AE8" s="246"/>
-      <c r="AF8" s="246"/>
-      <c r="AG8" s="246"/>
-      <c r="AH8" s="246"/>
-      <c r="AI8" s="246"/>
-      <c r="AJ8" s="246"/>
-      <c r="AK8" s="282"/>
-      <c r="AL8" s="246"/>
-      <c r="AM8" s="246"/>
-      <c r="AN8" s="246"/>
-      <c r="AO8" s="246"/>
-      <c r="AP8" s="246"/>
-      <c r="AQ8" s="246"/>
-      <c r="AR8" s="246"/>
-      <c r="AS8" s="246"/>
-      <c r="AT8" s="246"/>
-      <c r="AU8" s="246"/>
-      <c r="AV8" s="246"/>
-      <c r="AW8" s="246"/>
-      <c r="AX8" s="246"/>
+      <c r="X8" s="248"/>
+      <c r="Y8" s="248"/>
+      <c r="Z8" s="248"/>
+      <c r="AA8" s="248"/>
+      <c r="AB8" s="248"/>
+      <c r="AC8" s="248"/>
+      <c r="AD8" s="248"/>
+      <c r="AE8" s="248"/>
+      <c r="AF8" s="248"/>
+      <c r="AG8" s="248"/>
+      <c r="AH8" s="248"/>
+      <c r="AI8" s="248"/>
+      <c r="AJ8" s="248"/>
+      <c r="AK8" s="251"/>
+      <c r="AL8" s="248"/>
+      <c r="AM8" s="248"/>
+      <c r="AN8" s="248"/>
+      <c r="AO8" s="248"/>
+      <c r="AP8" s="248"/>
+      <c r="AQ8" s="248"/>
+      <c r="AR8" s="248"/>
+      <c r="AS8" s="248"/>
+      <c r="AT8" s="248"/>
+      <c r="AU8" s="248"/>
+      <c r="AV8" s="248"/>
+      <c r="AW8" s="248"/>
+      <c r="AX8" s="248"/>
       <c r="AY8" s="102" t="s">
         <v>88</v>
       </c>
@@ -11590,27 +11745,27 @@
       <c r="BA8" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="BB8" s="246"/>
-      <c r="BC8" s="246"/>
-      <c r="BD8" s="246"/>
-      <c r="BE8" s="246"/>
-      <c r="BF8" s="246"/>
-      <c r="BG8" s="246"/>
-      <c r="BH8" s="246"/>
-      <c r="BI8" s="246"/>
-      <c r="BJ8" s="246"/>
-      <c r="BK8" s="246"/>
-      <c r="BL8" s="246"/>
-      <c r="BM8" s="246"/>
-      <c r="BN8" s="246"/>
-      <c r="BO8" s="246"/>
-      <c r="BP8" s="246"/>
-      <c r="BQ8" s="246"/>
-      <c r="BR8" s="246"/>
-      <c r="BS8" s="246"/>
-      <c r="BT8" s="246"/>
-      <c r="BU8" s="282"/>
-      <c r="BW8" s="260"/>
+      <c r="BB8" s="248"/>
+      <c r="BC8" s="248"/>
+      <c r="BD8" s="248"/>
+      <c r="BE8" s="248"/>
+      <c r="BF8" s="248"/>
+      <c r="BG8" s="248"/>
+      <c r="BH8" s="248"/>
+      <c r="BI8" s="248"/>
+      <c r="BJ8" s="248"/>
+      <c r="BK8" s="248"/>
+      <c r="BL8" s="248"/>
+      <c r="BM8" s="248"/>
+      <c r="BN8" s="248"/>
+      <c r="BO8" s="248"/>
+      <c r="BP8" s="248"/>
+      <c r="BQ8" s="248"/>
+      <c r="BR8" s="248"/>
+      <c r="BS8" s="248"/>
+      <c r="BT8" s="248"/>
+      <c r="BU8" s="251"/>
+      <c r="BW8" s="285"/>
       <c r="BX8" s="72" t="s">
         <v>91</v>
       </c>
@@ -11623,9 +11778,9 @@
       <c r="CA8" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="CB8" s="267"/>
-      <c r="CC8" s="267"/>
-      <c r="CD8" s="267"/>
+      <c r="CB8" s="246"/>
+      <c r="CC8" s="246"/>
+      <c r="CD8" s="246"/>
       <c r="CE8" s="141"/>
       <c r="CF8" s="146"/>
       <c r="CH8" s="142"/>
@@ -14075,26 +14230,69 @@
       <c r="CC24" s="201"/>
       <c r="CD24" s="201"/>
     </row>
+    <row r="25" spans="1:87" ht="17">
+      <c r="O25" s="301" t="s">
+        <v>154</v>
+      </c>
+    </row>
     <row r="26" spans="1:87" ht="28">
-      <c r="BN26" s="300" t="s">
+      <c r="BN26" s="243" t="s">
         <v>151</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A9:CI14" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="82">
-    <mergeCell ref="CD5:CD8"/>
-    <mergeCell ref="BR6:BR8"/>
-    <mergeCell ref="AT5:AT8"/>
-    <mergeCell ref="L6:L8"/>
-    <mergeCell ref="BM7:BM8"/>
-    <mergeCell ref="Z6:Z8"/>
-    <mergeCell ref="BJ7:BJ8"/>
-    <mergeCell ref="BL7:BL8"/>
-    <mergeCell ref="AW5:AW8"/>
-    <mergeCell ref="AI6:AI8"/>
-    <mergeCell ref="BU5:BU8"/>
-    <mergeCell ref="BW5:BW8"/>
+    <mergeCell ref="BS6:BS8"/>
+    <mergeCell ref="BM6:BQ6"/>
+    <mergeCell ref="AC6:AC8"/>
+    <mergeCell ref="BC7:BC8"/>
+    <mergeCell ref="AE6:AE8"/>
+    <mergeCell ref="BK7:BK8"/>
+    <mergeCell ref="BQ7:BQ8"/>
+    <mergeCell ref="BN7:BN8"/>
+    <mergeCell ref="BP7:BP8"/>
+    <mergeCell ref="AM6:AM8"/>
+    <mergeCell ref="AP5:AP8"/>
+    <mergeCell ref="BO7:BO8"/>
+    <mergeCell ref="BB7:BB8"/>
+    <mergeCell ref="BD7:BD8"/>
+    <mergeCell ref="BF7:BF8"/>
+    <mergeCell ref="BH7:BH8"/>
+    <mergeCell ref="S6:S8"/>
+    <mergeCell ref="AS5:AS8"/>
+    <mergeCell ref="AU5:AU8"/>
+    <mergeCell ref="AB6:AB8"/>
+    <mergeCell ref="AH6:AH8"/>
+    <mergeCell ref="AJ6:AJ8"/>
+    <mergeCell ref="T6:T8"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="AK6:AK8"/>
+    <mergeCell ref="BI7:BI8"/>
+    <mergeCell ref="K5:X5"/>
+    <mergeCell ref="AO6:AO8"/>
+    <mergeCell ref="Y5:AO5"/>
+    <mergeCell ref="AN6:AN8"/>
+    <mergeCell ref="AR5:AR8"/>
+    <mergeCell ref="AA6:AA8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="X6:X8"/>
+    <mergeCell ref="AV5:AV8"/>
+    <mergeCell ref="AX5:AX8"/>
+    <mergeCell ref="V6:W7"/>
+    <mergeCell ref="Y6:Y8"/>
+    <mergeCell ref="G5:G8"/>
+    <mergeCell ref="AQ5:AQ8"/>
+    <mergeCell ref="I5:I8"/>
+    <mergeCell ref="R6:R8"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="AL6:AL8"/>
+    <mergeCell ref="P6:P8"/>
+    <mergeCell ref="N6:N8"/>
+    <mergeCell ref="F5:F8"/>
+    <mergeCell ref="M6:M8"/>
+    <mergeCell ref="Q6:Q8"/>
     <mergeCell ref="BW3:CB4"/>
     <mergeCell ref="CC5:CC8"/>
     <mergeCell ref="AY6:BL6"/>
@@ -14111,60 +14309,22 @@
     <mergeCell ref="A3:BU3"/>
     <mergeCell ref="E5:E8"/>
     <mergeCell ref="K6:K8"/>
+    <mergeCell ref="CD5:CD8"/>
+    <mergeCell ref="BR6:BR8"/>
+    <mergeCell ref="AT5:AT8"/>
+    <mergeCell ref="L6:L8"/>
+    <mergeCell ref="BM7:BM8"/>
+    <mergeCell ref="Z6:Z8"/>
+    <mergeCell ref="BJ7:BJ8"/>
+    <mergeCell ref="BL7:BL8"/>
+    <mergeCell ref="AW5:AW8"/>
+    <mergeCell ref="AI6:AI8"/>
+    <mergeCell ref="BU5:BU8"/>
+    <mergeCell ref="BW5:BW8"/>
     <mergeCell ref="O6:O8"/>
-    <mergeCell ref="G5:G8"/>
-    <mergeCell ref="AQ5:AQ8"/>
-    <mergeCell ref="I5:I8"/>
-    <mergeCell ref="R6:R8"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="C5:C8"/>
-    <mergeCell ref="AK6:AK8"/>
-    <mergeCell ref="BI7:BI8"/>
-    <mergeCell ref="K5:X5"/>
-    <mergeCell ref="AO6:AO8"/>
-    <mergeCell ref="Y5:AO5"/>
-    <mergeCell ref="AN6:AN8"/>
-    <mergeCell ref="AR5:AR8"/>
-    <mergeCell ref="AA6:AA8"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="X6:X8"/>
-    <mergeCell ref="AV5:AV8"/>
-    <mergeCell ref="AX5:AX8"/>
-    <mergeCell ref="V6:W7"/>
-    <mergeCell ref="Y6:Y8"/>
     <mergeCell ref="AY5:BQ5"/>
     <mergeCell ref="CB5:CB8"/>
     <mergeCell ref="BT5:BT8"/>
-    <mergeCell ref="AL6:AL8"/>
-    <mergeCell ref="P6:P8"/>
-    <mergeCell ref="BB7:BB8"/>
-    <mergeCell ref="BD7:BD8"/>
-    <mergeCell ref="BF7:BF8"/>
-    <mergeCell ref="BH7:BH8"/>
-    <mergeCell ref="S6:S8"/>
-    <mergeCell ref="AS5:AS8"/>
-    <mergeCell ref="AU5:AU8"/>
-    <mergeCell ref="BK7:BK8"/>
-    <mergeCell ref="BQ7:BQ8"/>
-    <mergeCell ref="BN7:BN8"/>
-    <mergeCell ref="BP7:BP8"/>
-    <mergeCell ref="AM6:AM8"/>
-    <mergeCell ref="N6:N8"/>
-    <mergeCell ref="F5:F8"/>
-    <mergeCell ref="AP5:AP8"/>
-    <mergeCell ref="BO7:BO8"/>
-    <mergeCell ref="AB6:AB8"/>
-    <mergeCell ref="M6:M8"/>
-    <mergeCell ref="AH6:AH8"/>
-    <mergeCell ref="AJ6:AJ8"/>
-    <mergeCell ref="T6:T8"/>
-    <mergeCell ref="Q6:Q8"/>
-    <mergeCell ref="BS6:BS8"/>
-    <mergeCell ref="BM6:BQ6"/>
-    <mergeCell ref="AC6:AC8"/>
-    <mergeCell ref="BC7:BC8"/>
-    <mergeCell ref="AE6:AE8"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B9 B12:B16 B20:B1048576 C9:BU9 D10:F10 J10:BK10 BM10:BU10 BW9:CD10">
     <cfRule type="duplicateValues" dxfId="19" priority="54"/>
@@ -14392,88 +14552,88 @@
       <c r="CD2" s="12"/>
     </row>
     <row r="3" spans="1:87" s="16" customFormat="1" ht="24" customHeight="1" outlineLevel="1">
-      <c r="A3" s="277"/>
-      <c r="B3" s="274"/>
-      <c r="C3" s="274"/>
-      <c r="D3" s="274"/>
-      <c r="E3" s="274"/>
-      <c r="F3" s="274"/>
-      <c r="G3" s="274"/>
-      <c r="H3" s="274"/>
-      <c r="I3" s="274"/>
-      <c r="J3" s="274"/>
-      <c r="K3" s="274"/>
-      <c r="L3" s="274"/>
-      <c r="M3" s="274"/>
-      <c r="N3" s="274"/>
-      <c r="O3" s="274"/>
-      <c r="P3" s="274"/>
-      <c r="Q3" s="274"/>
-      <c r="R3" s="274"/>
-      <c r="S3" s="274"/>
-      <c r="T3" s="274"/>
-      <c r="U3" s="274"/>
-      <c r="V3" s="274"/>
-      <c r="W3" s="274"/>
-      <c r="X3" s="274"/>
-      <c r="Y3" s="274"/>
-      <c r="Z3" s="274"/>
-      <c r="AA3" s="274"/>
-      <c r="AB3" s="274"/>
-      <c r="AC3" s="274"/>
-      <c r="AD3" s="274"/>
-      <c r="AE3" s="274"/>
-      <c r="AF3" s="274"/>
-      <c r="AG3" s="274"/>
-      <c r="AH3" s="274"/>
-      <c r="AI3" s="274"/>
-      <c r="AJ3" s="274"/>
-      <c r="AK3" s="274"/>
-      <c r="AL3" s="274"/>
-      <c r="AM3" s="274"/>
-      <c r="AN3" s="274"/>
-      <c r="AO3" s="274"/>
-      <c r="AP3" s="274"/>
-      <c r="AQ3" s="274"/>
-      <c r="AR3" s="274"/>
-      <c r="AS3" s="274"/>
-      <c r="AT3" s="274"/>
-      <c r="AU3" s="274"/>
-      <c r="AV3" s="274"/>
-      <c r="AW3" s="274"/>
-      <c r="AX3" s="274"/>
-      <c r="AY3" s="274"/>
-      <c r="AZ3" s="274"/>
-      <c r="BA3" s="274"/>
-      <c r="BB3" s="274"/>
-      <c r="BC3" s="274"/>
-      <c r="BD3" s="274"/>
-      <c r="BE3" s="274"/>
-      <c r="BF3" s="274"/>
-      <c r="BG3" s="274"/>
-      <c r="BH3" s="274"/>
-      <c r="BI3" s="274"/>
-      <c r="BJ3" s="274"/>
-      <c r="BK3" s="274"/>
-      <c r="BL3" s="274"/>
-      <c r="BM3" s="274"/>
-      <c r="BN3" s="274"/>
-      <c r="BO3" s="274"/>
-      <c r="BP3" s="274"/>
-      <c r="BQ3" s="274"/>
-      <c r="BR3" s="274"/>
-      <c r="BS3" s="274"/>
-      <c r="BT3" s="274"/>
-      <c r="BU3" s="274"/>
+      <c r="A3" s="268"/>
+      <c r="B3" s="266"/>
+      <c r="C3" s="266"/>
+      <c r="D3" s="266"/>
+      <c r="E3" s="266"/>
+      <c r="F3" s="266"/>
+      <c r="G3" s="266"/>
+      <c r="H3" s="266"/>
+      <c r="I3" s="266"/>
+      <c r="J3" s="266"/>
+      <c r="K3" s="266"/>
+      <c r="L3" s="266"/>
+      <c r="M3" s="266"/>
+      <c r="N3" s="266"/>
+      <c r="O3" s="266"/>
+      <c r="P3" s="266"/>
+      <c r="Q3" s="266"/>
+      <c r="R3" s="266"/>
+      <c r="S3" s="266"/>
+      <c r="T3" s="266"/>
+      <c r="U3" s="266"/>
+      <c r="V3" s="266"/>
+      <c r="W3" s="266"/>
+      <c r="X3" s="266"/>
+      <c r="Y3" s="266"/>
+      <c r="Z3" s="266"/>
+      <c r="AA3" s="266"/>
+      <c r="AB3" s="266"/>
+      <c r="AC3" s="266"/>
+      <c r="AD3" s="266"/>
+      <c r="AE3" s="266"/>
+      <c r="AF3" s="266"/>
+      <c r="AG3" s="266"/>
+      <c r="AH3" s="266"/>
+      <c r="AI3" s="266"/>
+      <c r="AJ3" s="266"/>
+      <c r="AK3" s="266"/>
+      <c r="AL3" s="266"/>
+      <c r="AM3" s="266"/>
+      <c r="AN3" s="266"/>
+      <c r="AO3" s="266"/>
+      <c r="AP3" s="266"/>
+      <c r="AQ3" s="266"/>
+      <c r="AR3" s="266"/>
+      <c r="AS3" s="266"/>
+      <c r="AT3" s="266"/>
+      <c r="AU3" s="266"/>
+      <c r="AV3" s="266"/>
+      <c r="AW3" s="266"/>
+      <c r="AX3" s="266"/>
+      <c r="AY3" s="266"/>
+      <c r="AZ3" s="266"/>
+      <c r="BA3" s="266"/>
+      <c r="BB3" s="266"/>
+      <c r="BC3" s="266"/>
+      <c r="BD3" s="266"/>
+      <c r="BE3" s="266"/>
+      <c r="BF3" s="266"/>
+      <c r="BG3" s="266"/>
+      <c r="BH3" s="266"/>
+      <c r="BI3" s="266"/>
+      <c r="BJ3" s="266"/>
+      <c r="BK3" s="266"/>
+      <c r="BL3" s="266"/>
+      <c r="BM3" s="266"/>
+      <c r="BN3" s="266"/>
+      <c r="BO3" s="266"/>
+      <c r="BP3" s="266"/>
+      <c r="BQ3" s="266"/>
+      <c r="BR3" s="266"/>
+      <c r="BS3" s="266"/>
+      <c r="BT3" s="266"/>
+      <c r="BU3" s="266"/>
       <c r="BV3" s="110"/>
-      <c r="BW3" s="273" t="s">
+      <c r="BW3" s="265" t="s">
         <v>2</v>
       </c>
-      <c r="BX3" s="274"/>
-      <c r="BY3" s="274"/>
-      <c r="BZ3" s="274"/>
-      <c r="CA3" s="274"/>
-      <c r="CB3" s="274"/>
+      <c r="BX3" s="266"/>
+      <c r="BY3" s="266"/>
+      <c r="BZ3" s="266"/>
+      <c r="CA3" s="266"/>
+      <c r="CB3" s="266"/>
       <c r="CC3" s="71"/>
       <c r="CD3" s="71"/>
       <c r="CE3" s="16" t="s">
@@ -14557,12 +14717,12 @@
       <c r="BT4" s="15"/>
       <c r="BU4" s="15"/>
       <c r="BV4" s="111"/>
-      <c r="BW4" s="274"/>
-      <c r="BX4" s="274"/>
-      <c r="BY4" s="274"/>
-      <c r="BZ4" s="274"/>
-      <c r="CA4" s="274"/>
-      <c r="CB4" s="274"/>
+      <c r="BW4" s="266"/>
+      <c r="BX4" s="266"/>
+      <c r="BY4" s="266"/>
+      <c r="BZ4" s="266"/>
+      <c r="CA4" s="266"/>
+      <c r="CB4" s="266"/>
       <c r="CC4" s="71"/>
       <c r="CD4" s="71"/>
     </row>
@@ -14640,12 +14800,12 @@
       <c r="BT5" s="15"/>
       <c r="BU5" s="15"/>
       <c r="BV5" s="111"/>
-      <c r="BW5" s="275"/>
-      <c r="BX5" s="275"/>
-      <c r="BY5" s="275"/>
-      <c r="BZ5" s="275"/>
-      <c r="CA5" s="275"/>
-      <c r="CB5" s="275"/>
+      <c r="BW5" s="267"/>
+      <c r="BX5" s="267"/>
+      <c r="BY5" s="267"/>
+      <c r="BZ5" s="267"/>
+      <c r="CA5" s="267"/>
+      <c r="CB5" s="267"/>
       <c r="CC5" s="71"/>
       <c r="CD5" s="71"/>
     </row>
@@ -14723,12 +14883,12 @@
       <c r="BT6" s="18"/>
       <c r="BU6" s="18"/>
       <c r="BV6" s="112"/>
-      <c r="BW6" s="275"/>
-      <c r="BX6" s="275"/>
-      <c r="BY6" s="275"/>
-      <c r="BZ6" s="275"/>
-      <c r="CA6" s="275"/>
-      <c r="CB6" s="275"/>
+      <c r="BW6" s="267"/>
+      <c r="BX6" s="267"/>
+      <c r="BY6" s="267"/>
+      <c r="BZ6" s="267"/>
+      <c r="CA6" s="267"/>
+      <c r="CB6" s="267"/>
       <c r="CC6" s="71"/>
       <c r="CD6" s="71"/>
     </row>
@@ -14816,358 +14976,358 @@
       <c r="CD7" s="25"/>
     </row>
     <row r="8" spans="1:87" s="11" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A8" s="251" t="s">
+      <c r="A8" s="278" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="279" t="s">
+      <c r="B8" s="271" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="261" t="s">
+      <c r="C8" s="252" t="s">
         <v>6</v>
       </c>
-      <c r="D8" s="263" t="s">
+      <c r="D8" s="255" t="s">
         <v>141</v>
       </c>
-      <c r="E8" s="263" t="s">
+      <c r="E8" s="255" t="s">
         <v>8</v>
       </c>
-      <c r="F8" s="297" t="s">
+      <c r="F8" s="299" t="s">
         <v>142</v>
       </c>
-      <c r="G8" s="242" t="s">
+      <c r="G8" s="256" t="s">
         <v>10</v>
       </c>
-      <c r="H8" s="270" t="s">
+      <c r="H8" s="262" t="s">
         <v>11</v>
       </c>
-      <c r="I8" s="270" t="s">
+      <c r="I8" s="262" t="s">
         <v>12</v>
       </c>
-      <c r="J8" s="242" t="s">
+      <c r="J8" s="256" t="s">
         <v>13</v>
       </c>
-      <c r="K8" s="271" t="s">
+      <c r="K8" s="276" t="s">
         <v>14</v>
       </c>
-      <c r="L8" s="243"/>
-      <c r="M8" s="243"/>
-      <c r="N8" s="243"/>
-      <c r="O8" s="243"/>
-      <c r="P8" s="243"/>
-      <c r="Q8" s="243"/>
-      <c r="R8" s="243"/>
-      <c r="S8" s="243"/>
-      <c r="T8" s="243"/>
-      <c r="U8" s="243"/>
-      <c r="V8" s="243"/>
-      <c r="W8" s="243"/>
-      <c r="X8" s="243"/>
-      <c r="Y8" s="242" t="s">
+      <c r="L8" s="273"/>
+      <c r="M8" s="273"/>
+      <c r="N8" s="273"/>
+      <c r="O8" s="273"/>
+      <c r="P8" s="273"/>
+      <c r="Q8" s="273"/>
+      <c r="R8" s="273"/>
+      <c r="S8" s="273"/>
+      <c r="T8" s="273"/>
+      <c r="U8" s="273"/>
+      <c r="V8" s="273"/>
+      <c r="W8" s="273"/>
+      <c r="X8" s="273"/>
+      <c r="Y8" s="256" t="s">
         <v>15</v>
       </c>
-      <c r="Z8" s="243"/>
-      <c r="AA8" s="243"/>
-      <c r="AB8" s="243"/>
-      <c r="AC8" s="243"/>
-      <c r="AD8" s="243"/>
-      <c r="AE8" s="243"/>
-      <c r="AF8" s="243"/>
-      <c r="AG8" s="243"/>
-      <c r="AH8" s="243"/>
-      <c r="AI8" s="243"/>
-      <c r="AJ8" s="243"/>
-      <c r="AK8" s="243"/>
-      <c r="AL8" s="243"/>
-      <c r="AM8" s="243"/>
-      <c r="AN8" s="243"/>
-      <c r="AO8" s="244"/>
-      <c r="AP8" s="242" t="s">
+      <c r="Z8" s="273"/>
+      <c r="AA8" s="273"/>
+      <c r="AB8" s="273"/>
+      <c r="AC8" s="273"/>
+      <c r="AD8" s="273"/>
+      <c r="AE8" s="273"/>
+      <c r="AF8" s="273"/>
+      <c r="AG8" s="273"/>
+      <c r="AH8" s="273"/>
+      <c r="AI8" s="273"/>
+      <c r="AJ8" s="273"/>
+      <c r="AK8" s="273"/>
+      <c r="AL8" s="273"/>
+      <c r="AM8" s="273"/>
+      <c r="AN8" s="273"/>
+      <c r="AO8" s="274"/>
+      <c r="AP8" s="256" t="s">
         <v>16</v>
       </c>
-      <c r="AQ8" s="242" t="s">
+      <c r="AQ8" s="256" t="s">
         <v>17</v>
       </c>
-      <c r="AR8" s="242" t="s">
+      <c r="AR8" s="256" t="s">
         <v>18</v>
       </c>
-      <c r="AS8" s="242" t="s">
+      <c r="AS8" s="256" t="s">
         <v>19</v>
       </c>
-      <c r="AT8" s="242" t="s">
+      <c r="AT8" s="256" t="s">
         <v>20</v>
       </c>
-      <c r="AU8" s="242" t="s">
+      <c r="AU8" s="256" t="s">
         <v>21</v>
       </c>
-      <c r="AV8" s="261" t="s">
+      <c r="AV8" s="252" t="s">
         <v>22</v>
       </c>
-      <c r="AW8" s="261" t="s">
+      <c r="AW8" s="252" t="s">
         <v>23</v>
       </c>
-      <c r="AX8" s="261" t="s">
+      <c r="AX8" s="252" t="s">
         <v>24</v>
       </c>
-      <c r="AY8" s="268" t="s">
+      <c r="AY8" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ8" s="243"/>
-      <c r="BA8" s="243"/>
-      <c r="BB8" s="243"/>
-      <c r="BC8" s="243"/>
-      <c r="BD8" s="243"/>
-      <c r="BE8" s="243"/>
-      <c r="BF8" s="243"/>
-      <c r="BG8" s="243"/>
-      <c r="BH8" s="243"/>
-      <c r="BI8" s="243"/>
-      <c r="BJ8" s="243"/>
-      <c r="BK8" s="243"/>
-      <c r="BL8" s="243"/>
-      <c r="BM8" s="243"/>
-      <c r="BN8" s="243"/>
-      <c r="BO8" s="243"/>
-      <c r="BP8" s="244"/>
-      <c r="BQ8" s="280" t="s">
+      <c r="AZ8" s="273"/>
+      <c r="BA8" s="273"/>
+      <c r="BB8" s="273"/>
+      <c r="BC8" s="273"/>
+      <c r="BD8" s="273"/>
+      <c r="BE8" s="273"/>
+      <c r="BF8" s="273"/>
+      <c r="BG8" s="273"/>
+      <c r="BH8" s="273"/>
+      <c r="BI8" s="273"/>
+      <c r="BJ8" s="273"/>
+      <c r="BK8" s="273"/>
+      <c r="BL8" s="273"/>
+      <c r="BM8" s="273"/>
+      <c r="BN8" s="273"/>
+      <c r="BO8" s="273"/>
+      <c r="BP8" s="274"/>
+      <c r="BQ8" s="253" t="s">
         <v>26</v>
       </c>
       <c r="BR8" s="254"/>
-      <c r="BS8" s="268" t="s">
+      <c r="BS8" s="261" t="s">
         <v>143</v>
       </c>
-      <c r="BT8" s="268" t="s">
+      <c r="BT8" s="261" t="s">
         <v>27</v>
       </c>
-      <c r="BU8" s="281" t="s">
+      <c r="BU8" s="257" t="s">
         <v>28</v>
       </c>
       <c r="BV8" s="114"/>
-      <c r="BW8" s="262" t="s">
+      <c r="BW8" s="286" t="s">
         <v>29</v>
       </c>
-      <c r="BX8" s="252" t="s">
+      <c r="BX8" s="279" t="s">
         <v>30</v>
       </c>
-      <c r="BY8" s="253"/>
-      <c r="BZ8" s="253"/>
+      <c r="BY8" s="280"/>
+      <c r="BZ8" s="280"/>
       <c r="CA8" s="254"/>
-      <c r="CB8" s="266" t="s">
+      <c r="CB8" s="272" t="s">
         <v>31</v>
       </c>
-      <c r="CC8" s="276" t="s">
+      <c r="CC8" s="244" t="s">
         <v>32</v>
       </c>
-      <c r="CD8" s="276" t="s">
+      <c r="CD8" s="244" t="s">
         <v>33</v>
       </c>
       <c r="CH8" s="27"/>
       <c r="CI8" s="28"/>
     </row>
     <row r="9" spans="1:87" s="11" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A9" s="248"/>
-      <c r="B9" s="248"/>
-      <c r="C9" s="248"/>
-      <c r="D9" s="248"/>
-      <c r="E9" s="248"/>
-      <c r="F9" s="248"/>
-      <c r="G9" s="248"/>
-      <c r="H9" s="248"/>
-      <c r="I9" s="248"/>
-      <c r="J9" s="248"/>
-      <c r="K9" s="247" t="s">
+      <c r="A9" s="245"/>
+      <c r="B9" s="245"/>
+      <c r="C9" s="245"/>
+      <c r="D9" s="245"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="245"/>
+      <c r="G9" s="245"/>
+      <c r="H9" s="245"/>
+      <c r="I9" s="245"/>
+      <c r="J9" s="245"/>
+      <c r="K9" s="258" t="s">
         <v>34</v>
       </c>
-      <c r="L9" s="247" t="s">
+      <c r="L9" s="258" t="s">
         <v>35</v>
       </c>
-      <c r="M9" s="247" t="s">
+      <c r="M9" s="258" t="s">
         <v>36</v>
       </c>
-      <c r="N9" s="247" t="s">
+      <c r="N9" s="258" t="s">
         <v>37</v>
       </c>
-      <c r="O9" s="247" t="s">
+      <c r="O9" s="258" t="s">
         <v>38</v>
       </c>
-      <c r="P9" s="247" t="s">
+      <c r="P9" s="258" t="s">
         <v>39</v>
       </c>
-      <c r="Q9" s="247" t="s">
+      <c r="Q9" s="258" t="s">
         <v>40</v>
       </c>
-      <c r="R9" s="247" t="s">
+      <c r="R9" s="258" t="s">
         <v>41</v>
       </c>
-      <c r="S9" s="247" t="s">
+      <c r="S9" s="258" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="247" t="s">
+      <c r="T9" s="258" t="s">
         <v>43</v>
       </c>
-      <c r="U9" s="247" t="s">
+      <c r="U9" s="258" t="s">
         <v>44</v>
       </c>
-      <c r="V9" s="284" t="s">
+      <c r="V9" s="263" t="s">
         <v>45</v>
       </c>
       <c r="W9" s="254"/>
-      <c r="X9" s="247" t="s">
+      <c r="X9" s="258" t="s">
         <v>46</v>
       </c>
-      <c r="Y9" s="249" t="s">
+      <c r="Y9" s="247" t="s">
         <v>47</v>
       </c>
-      <c r="Z9" s="249" t="s">
+      <c r="Z9" s="247" t="s">
         <v>48</v>
       </c>
-      <c r="AA9" s="249" t="s">
+      <c r="AA9" s="247" t="s">
         <v>49</v>
       </c>
-      <c r="AB9" s="249" t="s">
+      <c r="AB9" s="247" t="s">
         <v>50</v>
       </c>
-      <c r="AC9" s="250" t="s">
+      <c r="AC9" s="269" t="s">
         <v>51</v>
       </c>
-      <c r="AD9" s="250" t="s">
+      <c r="AD9" s="269" t="s">
         <v>144</v>
       </c>
-      <c r="AE9" s="250" t="s">
+      <c r="AE9" s="269" t="s">
         <v>53</v>
       </c>
-      <c r="AF9" s="250" t="s">
+      <c r="AF9" s="269" t="s">
         <v>54</v>
       </c>
-      <c r="AG9" s="249" t="s">
+      <c r="AG9" s="247" t="s">
         <v>55</v>
       </c>
-      <c r="AH9" s="250" t="s">
+      <c r="AH9" s="269" t="s">
         <v>56</v>
       </c>
-      <c r="AI9" s="250" t="s">
+      <c r="AI9" s="269" t="s">
         <v>57</v>
       </c>
-      <c r="AJ9" s="249" t="s">
+      <c r="AJ9" s="247" t="s">
         <v>58</v>
       </c>
-      <c r="AK9" s="283" t="s">
+      <c r="AK9" s="249" t="s">
         <v>59</v>
       </c>
-      <c r="AL9" s="261" t="s">
+      <c r="AL9" s="252" t="s">
         <v>60</v>
       </c>
-      <c r="AM9" s="249" t="s">
+      <c r="AM9" s="247" t="s">
         <v>61</v>
       </c>
-      <c r="AN9" s="269" t="s">
+      <c r="AN9" s="275" t="s">
         <v>62</v>
       </c>
-      <c r="AO9" s="261" t="s">
+      <c r="AO9" s="252" t="s">
         <v>63</v>
       </c>
-      <c r="AP9" s="248"/>
-      <c r="AQ9" s="248"/>
-      <c r="AR9" s="248"/>
-      <c r="AS9" s="248"/>
-      <c r="AT9" s="248"/>
-      <c r="AU9" s="248"/>
-      <c r="AV9" s="248"/>
-      <c r="AW9" s="248"/>
-      <c r="AX9" s="248"/>
-      <c r="AY9" s="268" t="s">
+      <c r="AP9" s="245"/>
+      <c r="AQ9" s="245"/>
+      <c r="AR9" s="245"/>
+      <c r="AS9" s="245"/>
+      <c r="AT9" s="245"/>
+      <c r="AU9" s="245"/>
+      <c r="AV9" s="245"/>
+      <c r="AW9" s="245"/>
+      <c r="AX9" s="245"/>
+      <c r="AY9" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ9" s="243"/>
-      <c r="BA9" s="243"/>
-      <c r="BB9" s="243"/>
-      <c r="BC9" s="243"/>
-      <c r="BD9" s="243"/>
-      <c r="BE9" s="243"/>
-      <c r="BF9" s="243"/>
-      <c r="BG9" s="243"/>
-      <c r="BH9" s="243"/>
-      <c r="BI9" s="243"/>
-      <c r="BJ9" s="244"/>
-      <c r="BK9" s="268" t="s">
+      <c r="AZ9" s="273"/>
+      <c r="BA9" s="273"/>
+      <c r="BB9" s="273"/>
+      <c r="BC9" s="273"/>
+      <c r="BD9" s="273"/>
+      <c r="BE9" s="273"/>
+      <c r="BF9" s="273"/>
+      <c r="BG9" s="273"/>
+      <c r="BH9" s="273"/>
+      <c r="BI9" s="273"/>
+      <c r="BJ9" s="274"/>
+      <c r="BK9" s="261" t="s">
         <v>64</v>
       </c>
-      <c r="BL9" s="243"/>
-      <c r="BM9" s="243"/>
-      <c r="BN9" s="243"/>
-      <c r="BO9" s="243"/>
-      <c r="BP9" s="244"/>
-      <c r="BQ9" s="265" t="s">
+      <c r="BL9" s="273"/>
+      <c r="BM9" s="273"/>
+      <c r="BN9" s="273"/>
+      <c r="BO9" s="273"/>
+      <c r="BP9" s="274"/>
+      <c r="BQ9" s="259" t="s">
         <v>65</v>
       </c>
-      <c r="BR9" s="265" t="s">
+      <c r="BR9" s="259" t="s">
         <v>66</v>
       </c>
-      <c r="BS9" s="248"/>
-      <c r="BT9" s="248"/>
-      <c r="BU9" s="255"/>
+      <c r="BS9" s="245"/>
+      <c r="BT9" s="245"/>
+      <c r="BU9" s="250"/>
       <c r="BV9" s="114"/>
-      <c r="BW9" s="257"/>
-      <c r="BX9" s="255"/>
-      <c r="BY9" s="256"/>
-      <c r="BZ9" s="256"/>
-      <c r="CA9" s="257"/>
-      <c r="CB9" s="248"/>
-      <c r="CC9" s="248"/>
-      <c r="CD9" s="248"/>
+      <c r="BW9" s="282"/>
+      <c r="BX9" s="250"/>
+      <c r="BY9" s="281"/>
+      <c r="BZ9" s="281"/>
+      <c r="CA9" s="282"/>
+      <c r="CB9" s="245"/>
+      <c r="CC9" s="245"/>
+      <c r="CD9" s="245"/>
       <c r="CH9" s="27"/>
       <c r="CI9" s="28"/>
     </row>
     <row r="10" spans="1:87" s="29" customFormat="1" ht="19.25" customHeight="1">
-      <c r="A10" s="248"/>
-      <c r="B10" s="248"/>
-      <c r="C10" s="248"/>
-      <c r="D10" s="248"/>
-      <c r="E10" s="248"/>
-      <c r="F10" s="248"/>
-      <c r="G10" s="248"/>
-      <c r="H10" s="248"/>
-      <c r="I10" s="248"/>
-      <c r="J10" s="248"/>
-      <c r="K10" s="248"/>
-      <c r="L10" s="248"/>
-      <c r="M10" s="248"/>
-      <c r="N10" s="248"/>
-      <c r="O10" s="248"/>
-      <c r="P10" s="248"/>
-      <c r="Q10" s="248"/>
-      <c r="R10" s="248"/>
-      <c r="S10" s="248"/>
-      <c r="T10" s="248"/>
-      <c r="U10" s="248"/>
-      <c r="V10" s="282"/>
-      <c r="W10" s="285"/>
-      <c r="X10" s="248"/>
-      <c r="Y10" s="248"/>
-      <c r="Z10" s="248"/>
-      <c r="AA10" s="248"/>
-      <c r="AB10" s="248"/>
-      <c r="AC10" s="248"/>
-      <c r="AD10" s="248"/>
-      <c r="AE10" s="248"/>
-      <c r="AF10" s="248"/>
-      <c r="AG10" s="248"/>
-      <c r="AH10" s="248"/>
-      <c r="AI10" s="248"/>
-      <c r="AJ10" s="248"/>
-      <c r="AK10" s="255"/>
-      <c r="AL10" s="248"/>
-      <c r="AM10" s="248"/>
-      <c r="AN10" s="248"/>
-      <c r="AO10" s="248"/>
-      <c r="AP10" s="248"/>
-      <c r="AQ10" s="248"/>
-      <c r="AR10" s="248"/>
-      <c r="AS10" s="248"/>
-      <c r="AT10" s="248"/>
-      <c r="AU10" s="248"/>
-      <c r="AV10" s="248"/>
-      <c r="AW10" s="248"/>
-      <c r="AX10" s="248"/>
+      <c r="A10" s="245"/>
+      <c r="B10" s="245"/>
+      <c r="C10" s="245"/>
+      <c r="D10" s="245"/>
+      <c r="E10" s="245"/>
+      <c r="F10" s="245"/>
+      <c r="G10" s="245"/>
+      <c r="H10" s="245"/>
+      <c r="I10" s="245"/>
+      <c r="J10" s="245"/>
+      <c r="K10" s="245"/>
+      <c r="L10" s="245"/>
+      <c r="M10" s="245"/>
+      <c r="N10" s="245"/>
+      <c r="O10" s="245"/>
+      <c r="P10" s="245"/>
+      <c r="Q10" s="245"/>
+      <c r="R10" s="245"/>
+      <c r="S10" s="245"/>
+      <c r="T10" s="245"/>
+      <c r="U10" s="245"/>
+      <c r="V10" s="251"/>
+      <c r="W10" s="264"/>
+      <c r="X10" s="245"/>
+      <c r="Y10" s="245"/>
+      <c r="Z10" s="245"/>
+      <c r="AA10" s="245"/>
+      <c r="AB10" s="245"/>
+      <c r="AC10" s="245"/>
+      <c r="AD10" s="245"/>
+      <c r="AE10" s="245"/>
+      <c r="AF10" s="245"/>
+      <c r="AG10" s="245"/>
+      <c r="AH10" s="245"/>
+      <c r="AI10" s="245"/>
+      <c r="AJ10" s="245"/>
+      <c r="AK10" s="250"/>
+      <c r="AL10" s="245"/>
+      <c r="AM10" s="245"/>
+      <c r="AN10" s="245"/>
+      <c r="AO10" s="245"/>
+      <c r="AP10" s="245"/>
+      <c r="AQ10" s="245"/>
+      <c r="AR10" s="245"/>
+      <c r="AS10" s="245"/>
+      <c r="AT10" s="245"/>
+      <c r="AU10" s="245"/>
+      <c r="AV10" s="245"/>
+      <c r="AW10" s="245"/>
+      <c r="AX10" s="245"/>
       <c r="AY10" s="101" t="s">
         <v>67</v>
       </c>
@@ -15180,120 +15340,120 @@
       <c r="BB10" s="298" t="s">
         <v>70</v>
       </c>
-      <c r="BC10" s="295" t="s">
+      <c r="BC10" s="296" t="s">
         <v>71</v>
       </c>
-      <c r="BD10" s="295" t="s">
+      <c r="BD10" s="296" t="s">
         <v>72</v>
       </c>
-      <c r="BE10" s="295" t="s">
+      <c r="BE10" s="296" t="s">
         <v>145</v>
       </c>
-      <c r="BF10" s="295" t="s">
+      <c r="BF10" s="296" t="s">
         <v>74</v>
       </c>
-      <c r="BG10" s="295" t="s">
+      <c r="BG10" s="296" t="s">
         <v>75</v>
       </c>
-      <c r="BH10" s="295" t="s">
+      <c r="BH10" s="296" t="s">
         <v>76</v>
       </c>
-      <c r="BI10" s="295" t="s">
+      <c r="BI10" s="296" t="s">
         <v>79</v>
       </c>
-      <c r="BJ10" s="294" t="s">
+      <c r="BJ10" s="300" t="s">
         <v>80</v>
       </c>
-      <c r="BK10" s="295" t="s">
+      <c r="BK10" s="296" t="s">
         <v>81</v>
       </c>
-      <c r="BL10" s="296" t="s">
+      <c r="BL10" s="297" t="s">
         <v>82</v>
       </c>
-      <c r="BM10" s="295" t="s">
+      <c r="BM10" s="296" t="s">
         <v>83</v>
       </c>
-      <c r="BN10" s="296" t="s">
+      <c r="BN10" s="297" t="s">
         <v>84</v>
       </c>
-      <c r="BO10" s="296" t="s">
+      <c r="BO10" s="297" t="s">
         <v>146</v>
       </c>
-      <c r="BP10" s="268" t="s">
+      <c r="BP10" s="261" t="s">
         <v>85</v>
       </c>
-      <c r="BQ10" s="248"/>
-      <c r="BR10" s="248"/>
-      <c r="BS10" s="248"/>
-      <c r="BT10" s="248"/>
-      <c r="BU10" s="255"/>
+      <c r="BQ10" s="245"/>
+      <c r="BR10" s="245"/>
+      <c r="BS10" s="245"/>
+      <c r="BT10" s="245"/>
+      <c r="BU10" s="250"/>
       <c r="BV10" s="114"/>
-      <c r="BW10" s="257"/>
-      <c r="BX10" s="258"/>
-      <c r="BY10" s="259"/>
-      <c r="BZ10" s="259"/>
-      <c r="CA10" s="260"/>
-      <c r="CB10" s="248"/>
-      <c r="CC10" s="248"/>
-      <c r="CD10" s="248"/>
+      <c r="BW10" s="282"/>
+      <c r="BX10" s="283"/>
+      <c r="BY10" s="284"/>
+      <c r="BZ10" s="284"/>
+      <c r="CA10" s="285"/>
+      <c r="CB10" s="245"/>
+      <c r="CC10" s="245"/>
+      <c r="CD10" s="245"/>
       <c r="CH10" s="27"/>
       <c r="CI10" s="28"/>
     </row>
     <row r="11" spans="1:87" s="29" customFormat="1" ht="38.25" customHeight="1">
-      <c r="A11" s="246"/>
-      <c r="B11" s="246"/>
-      <c r="C11" s="246"/>
-      <c r="D11" s="246"/>
-      <c r="E11" s="246"/>
-      <c r="F11" s="246"/>
-      <c r="G11" s="246"/>
-      <c r="H11" s="246"/>
-      <c r="I11" s="246"/>
-      <c r="J11" s="246"/>
-      <c r="K11" s="246"/>
-      <c r="L11" s="246"/>
-      <c r="M11" s="246"/>
-      <c r="N11" s="246"/>
-      <c r="O11" s="246"/>
-      <c r="P11" s="246"/>
-      <c r="Q11" s="246"/>
-      <c r="R11" s="246"/>
-      <c r="S11" s="246"/>
-      <c r="T11" s="246"/>
-      <c r="U11" s="246"/>
+      <c r="A11" s="248"/>
+      <c r="B11" s="248"/>
+      <c r="C11" s="248"/>
+      <c r="D11" s="248"/>
+      <c r="E11" s="248"/>
+      <c r="F11" s="248"/>
+      <c r="G11" s="248"/>
+      <c r="H11" s="248"/>
+      <c r="I11" s="248"/>
+      <c r="J11" s="248"/>
+      <c r="K11" s="248"/>
+      <c r="L11" s="248"/>
+      <c r="M11" s="248"/>
+      <c r="N11" s="248"/>
+      <c r="O11" s="248"/>
+      <c r="P11" s="248"/>
+      <c r="Q11" s="248"/>
+      <c r="R11" s="248"/>
+      <c r="S11" s="248"/>
+      <c r="T11" s="248"/>
+      <c r="U11" s="248"/>
       <c r="V11" s="30" t="s">
         <v>86</v>
       </c>
       <c r="W11" s="30" t="s">
         <v>87</v>
       </c>
-      <c r="X11" s="246"/>
-      <c r="Y11" s="246"/>
-      <c r="Z11" s="246"/>
-      <c r="AA11" s="246"/>
-      <c r="AB11" s="246"/>
-      <c r="AC11" s="246"/>
-      <c r="AD11" s="246"/>
-      <c r="AE11" s="246"/>
-      <c r="AF11" s="246"/>
-      <c r="AG11" s="246"/>
-      <c r="AH11" s="246"/>
-      <c r="AI11" s="246"/>
-      <c r="AJ11" s="246"/>
-      <c r="AK11" s="282"/>
-      <c r="AL11" s="246"/>
-      <c r="AM11" s="246"/>
-      <c r="AN11" s="246"/>
-      <c r="AO11" s="246"/>
-      <c r="AP11" s="246"/>
-      <c r="AQ11" s="246"/>
-      <c r="AR11" s="246"/>
-      <c r="AS11" s="246"/>
-      <c r="AT11" s="246"/>
-      <c r="AU11" s="246"/>
-      <c r="AV11" s="246"/>
-      <c r="AW11" s="246"/>
-      <c r="AX11" s="246"/>
+      <c r="X11" s="248"/>
+      <c r="Y11" s="248"/>
+      <c r="Z11" s="248"/>
+      <c r="AA11" s="248"/>
+      <c r="AB11" s="248"/>
+      <c r="AC11" s="248"/>
+      <c r="AD11" s="248"/>
+      <c r="AE11" s="248"/>
+      <c r="AF11" s="248"/>
+      <c r="AG11" s="248"/>
+      <c r="AH11" s="248"/>
+      <c r="AI11" s="248"/>
+      <c r="AJ11" s="248"/>
+      <c r="AK11" s="251"/>
+      <c r="AL11" s="248"/>
+      <c r="AM11" s="248"/>
+      <c r="AN11" s="248"/>
+      <c r="AO11" s="248"/>
+      <c r="AP11" s="248"/>
+      <c r="AQ11" s="248"/>
+      <c r="AR11" s="248"/>
+      <c r="AS11" s="248"/>
+      <c r="AT11" s="248"/>
+      <c r="AU11" s="248"/>
+      <c r="AV11" s="248"/>
+      <c r="AW11" s="248"/>
+      <c r="AX11" s="248"/>
       <c r="AY11" s="102" t="s">
         <v>88</v>
       </c>
@@ -15303,28 +15463,28 @@
       <c r="BA11" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="BB11" s="246"/>
-      <c r="BC11" s="246"/>
-      <c r="BD11" s="246"/>
-      <c r="BE11" s="246"/>
-      <c r="BF11" s="246"/>
-      <c r="BG11" s="246"/>
-      <c r="BH11" s="246"/>
-      <c r="BI11" s="246"/>
-      <c r="BJ11" s="246"/>
-      <c r="BK11" s="246"/>
-      <c r="BL11" s="246"/>
-      <c r="BM11" s="246"/>
-      <c r="BN11" s="246"/>
-      <c r="BO11" s="246"/>
-      <c r="BP11" s="246"/>
-      <c r="BQ11" s="246"/>
-      <c r="BR11" s="246"/>
-      <c r="BS11" s="246"/>
-      <c r="BT11" s="246"/>
-      <c r="BU11" s="282"/>
+      <c r="BB11" s="248"/>
+      <c r="BC11" s="248"/>
+      <c r="BD11" s="248"/>
+      <c r="BE11" s="248"/>
+      <c r="BF11" s="248"/>
+      <c r="BG11" s="248"/>
+      <c r="BH11" s="248"/>
+      <c r="BI11" s="248"/>
+      <c r="BJ11" s="248"/>
+      <c r="BK11" s="248"/>
+      <c r="BL11" s="248"/>
+      <c r="BM11" s="248"/>
+      <c r="BN11" s="248"/>
+      <c r="BO11" s="248"/>
+      <c r="BP11" s="248"/>
+      <c r="BQ11" s="248"/>
+      <c r="BR11" s="248"/>
+      <c r="BS11" s="248"/>
+      <c r="BT11" s="248"/>
+      <c r="BU11" s="251"/>
       <c r="BV11" s="114"/>
-      <c r="BW11" s="260"/>
+      <c r="BW11" s="285"/>
       <c r="BX11" s="72" t="s">
         <v>91</v>
       </c>
@@ -15337,9 +15497,9 @@
       <c r="CA11" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="CB11" s="267"/>
-      <c r="CC11" s="267"/>
-      <c r="CD11" s="267"/>
+      <c r="CB11" s="246"/>
+      <c r="CC11" s="246"/>
+      <c r="CD11" s="246"/>
       <c r="CE11" s="11"/>
       <c r="CF11" s="31"/>
       <c r="CH11" s="27"/>
@@ -17723,7 +17883,7 @@
       <c r="CF24" s="57"/>
     </row>
     <row r="25" spans="1:87" ht="15" customHeight="1">
-      <c r="D25" s="299" t="s">
+      <c r="D25" s="242" t="s">
         <v>152</v>
       </c>
       <c r="I25" s="70"/>
@@ -17740,12 +17900,64 @@
   </sheetData>
   <autoFilter ref="A12:CI21" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <mergeCells count="82">
-    <mergeCell ref="CD8:CD11"/>
-    <mergeCell ref="Y9:Y11"/>
-    <mergeCell ref="AA9:AA11"/>
-    <mergeCell ref="AK9:AK11"/>
-    <mergeCell ref="AM9:AM11"/>
-    <mergeCell ref="AX8:AX11"/>
+    <mergeCell ref="L9:L11"/>
+    <mergeCell ref="N9:N11"/>
+    <mergeCell ref="BG10:BG11"/>
+    <mergeCell ref="BI10:BI11"/>
+    <mergeCell ref="X9:X11"/>
+    <mergeCell ref="Z9:Z11"/>
+    <mergeCell ref="AD9:AD11"/>
+    <mergeCell ref="AY9:BJ9"/>
+    <mergeCell ref="AT8:AT11"/>
+    <mergeCell ref="AV8:AV11"/>
+    <mergeCell ref="A8:A11"/>
+    <mergeCell ref="AS8:AS11"/>
+    <mergeCell ref="BX8:CA10"/>
+    <mergeCell ref="C8:C11"/>
+    <mergeCell ref="BW8:BW11"/>
+    <mergeCell ref="AI9:AI11"/>
+    <mergeCell ref="BQ8:BR8"/>
+    <mergeCell ref="D8:D11"/>
+    <mergeCell ref="BF10:BF11"/>
+    <mergeCell ref="BO10:BO11"/>
+    <mergeCell ref="Q9:Q11"/>
+    <mergeCell ref="S9:S11"/>
+    <mergeCell ref="BL10:BL11"/>
+    <mergeCell ref="AC9:AC11"/>
+    <mergeCell ref="AP8:AP11"/>
+    <mergeCell ref="AR8:AR11"/>
+    <mergeCell ref="F8:F11"/>
+    <mergeCell ref="CB8:CB11"/>
+    <mergeCell ref="AJ9:AJ11"/>
+    <mergeCell ref="AL9:AL11"/>
+    <mergeCell ref="AN9:AN11"/>
+    <mergeCell ref="I8:I11"/>
+    <mergeCell ref="BK10:BK11"/>
+    <mergeCell ref="K8:X8"/>
+    <mergeCell ref="BC10:BC11"/>
+    <mergeCell ref="BE10:BE11"/>
+    <mergeCell ref="T9:T11"/>
+    <mergeCell ref="P9:P11"/>
+    <mergeCell ref="AB9:AB11"/>
+    <mergeCell ref="AY8:BP8"/>
+    <mergeCell ref="AF9:AF11"/>
+    <mergeCell ref="AH9:AH11"/>
+    <mergeCell ref="BW3:CB6"/>
+    <mergeCell ref="AU8:AU11"/>
+    <mergeCell ref="CC8:CC11"/>
+    <mergeCell ref="AW8:AW11"/>
+    <mergeCell ref="A3:BU3"/>
+    <mergeCell ref="AE9:AE11"/>
+    <mergeCell ref="AO9:AO11"/>
+    <mergeCell ref="B8:B11"/>
+    <mergeCell ref="BB10:BB11"/>
+    <mergeCell ref="BD10:BD11"/>
+    <mergeCell ref="K9:K11"/>
+    <mergeCell ref="M9:M11"/>
+    <mergeCell ref="O9:O11"/>
+    <mergeCell ref="BH10:BH11"/>
+    <mergeCell ref="BQ9:BQ11"/>
+    <mergeCell ref="BT8:BT11"/>
     <mergeCell ref="E8:E11"/>
     <mergeCell ref="G8:G11"/>
     <mergeCell ref="BS8:BS11"/>
@@ -17762,66 +17974,14 @@
     <mergeCell ref="H8:H11"/>
     <mergeCell ref="J8:J11"/>
     <mergeCell ref="V9:W10"/>
-    <mergeCell ref="BW3:CB6"/>
-    <mergeCell ref="AU8:AU11"/>
-    <mergeCell ref="CC8:CC11"/>
-    <mergeCell ref="AW8:AW11"/>
-    <mergeCell ref="A3:BU3"/>
-    <mergeCell ref="AE9:AE11"/>
-    <mergeCell ref="AO9:AO11"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="BB10:BB11"/>
-    <mergeCell ref="BD10:BD11"/>
-    <mergeCell ref="K9:K11"/>
-    <mergeCell ref="M9:M11"/>
-    <mergeCell ref="O9:O11"/>
-    <mergeCell ref="BH10:BH11"/>
-    <mergeCell ref="BQ9:BQ11"/>
-    <mergeCell ref="BT8:BT11"/>
-    <mergeCell ref="F8:F11"/>
-    <mergeCell ref="CB8:CB11"/>
-    <mergeCell ref="AJ9:AJ11"/>
-    <mergeCell ref="AL9:AL11"/>
-    <mergeCell ref="AN9:AN11"/>
-    <mergeCell ref="I8:I11"/>
-    <mergeCell ref="BK10:BK11"/>
-    <mergeCell ref="K8:X8"/>
-    <mergeCell ref="BC10:BC11"/>
-    <mergeCell ref="BE10:BE11"/>
-    <mergeCell ref="T9:T11"/>
-    <mergeCell ref="P9:P11"/>
-    <mergeCell ref="AB9:AB11"/>
-    <mergeCell ref="AY8:BP8"/>
-    <mergeCell ref="AF9:AF11"/>
-    <mergeCell ref="AH9:AH11"/>
-    <mergeCell ref="A8:A11"/>
-    <mergeCell ref="AS8:AS11"/>
-    <mergeCell ref="BX8:CA10"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="BW8:BW11"/>
-    <mergeCell ref="AI9:AI11"/>
-    <mergeCell ref="BQ8:BR8"/>
-    <mergeCell ref="D8:D11"/>
-    <mergeCell ref="BF10:BF11"/>
-    <mergeCell ref="BO10:BO11"/>
-    <mergeCell ref="Q9:Q11"/>
-    <mergeCell ref="S9:S11"/>
-    <mergeCell ref="BL10:BL11"/>
-    <mergeCell ref="AC9:AC11"/>
-    <mergeCell ref="AP8:AP11"/>
-    <mergeCell ref="AR8:AR11"/>
+    <mergeCell ref="CD8:CD11"/>
+    <mergeCell ref="Y9:Y11"/>
+    <mergeCell ref="AA9:AA11"/>
+    <mergeCell ref="AK9:AK11"/>
+    <mergeCell ref="AM9:AM11"/>
+    <mergeCell ref="AX8:AX11"/>
     <mergeCell ref="Y8:AO8"/>
     <mergeCell ref="BJ10:BJ11"/>
-    <mergeCell ref="L9:L11"/>
-    <mergeCell ref="N9:N11"/>
-    <mergeCell ref="BG10:BG11"/>
-    <mergeCell ref="BI10:BI11"/>
-    <mergeCell ref="X9:X11"/>
-    <mergeCell ref="Z9:Z11"/>
-    <mergeCell ref="AD9:AD11"/>
-    <mergeCell ref="AY9:BJ9"/>
-    <mergeCell ref="AT8:AT11"/>
-    <mergeCell ref="AV8:AV11"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B12 B22:B1048576 C12:BU12">
     <cfRule type="duplicateValues" dxfId="12" priority="6"/>
@@ -18051,7 +18211,7 @@
       <c r="CD2" s="137"/>
     </row>
     <row r="3" spans="1:87" s="139" customFormat="1" ht="11" outlineLevel="1">
-      <c r="A3" s="290"/>
+      <c r="A3" s="293"/>
       <c r="B3" s="291"/>
       <c r="C3" s="291"/>
       <c r="D3" s="291"/>
@@ -18124,7 +18284,7 @@
       <c r="BS3" s="291"/>
       <c r="BT3" s="291"/>
       <c r="BU3" s="291"/>
-      <c r="BW3" s="293" t="s">
+      <c r="BW3" s="290" t="s">
         <v>2</v>
       </c>
       <c r="BX3" s="291"/>
@@ -18224,356 +18384,356 @@
       <c r="CD4" s="138"/>
     </row>
     <row r="5" spans="1:87" s="141" customFormat="1">
-      <c r="A5" s="251" t="s">
+      <c r="A5" s="278" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="279" t="s">
+      <c r="B5" s="271" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="261" t="s">
+      <c r="C5" s="252" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="263" t="s">
+      <c r="D5" s="255" t="s">
         <v>141</v>
       </c>
-      <c r="E5" s="263" t="s">
+      <c r="E5" s="255" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="297" t="s">
+      <c r="F5" s="299" t="s">
         <v>142</v>
       </c>
-      <c r="G5" s="261" t="s">
+      <c r="G5" s="252" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="287" t="s">
+      <c r="H5" s="289" t="s">
         <v>11</v>
       </c>
-      <c r="I5" s="287" t="s">
+      <c r="I5" s="289" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="261" t="s">
+      <c r="J5" s="252" t="s">
         <v>13</v>
       </c>
-      <c r="K5" s="288" t="s">
+      <c r="K5" s="294" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="243"/>
-      <c r="M5" s="243"/>
-      <c r="N5" s="243"/>
-      <c r="O5" s="243"/>
-      <c r="P5" s="243"/>
-      <c r="Q5" s="243"/>
-      <c r="R5" s="243"/>
-      <c r="S5" s="243"/>
-      <c r="T5" s="243"/>
-      <c r="U5" s="243"/>
-      <c r="V5" s="243"/>
-      <c r="W5" s="243"/>
-      <c r="X5" s="243"/>
-      <c r="Y5" s="261" t="s">
+      <c r="L5" s="273"/>
+      <c r="M5" s="273"/>
+      <c r="N5" s="273"/>
+      <c r="O5" s="273"/>
+      <c r="P5" s="273"/>
+      <c r="Q5" s="273"/>
+      <c r="R5" s="273"/>
+      <c r="S5" s="273"/>
+      <c r="T5" s="273"/>
+      <c r="U5" s="273"/>
+      <c r="V5" s="273"/>
+      <c r="W5" s="273"/>
+      <c r="X5" s="273"/>
+      <c r="Y5" s="252" t="s">
         <v>15</v>
       </c>
-      <c r="Z5" s="243"/>
-      <c r="AA5" s="243"/>
-      <c r="AB5" s="243"/>
-      <c r="AC5" s="243"/>
-      <c r="AD5" s="243"/>
-      <c r="AE5" s="243"/>
-      <c r="AF5" s="243"/>
-      <c r="AG5" s="243"/>
-      <c r="AH5" s="243"/>
-      <c r="AI5" s="243"/>
-      <c r="AJ5" s="243"/>
-      <c r="AK5" s="243"/>
-      <c r="AL5" s="243"/>
-      <c r="AM5" s="243"/>
-      <c r="AN5" s="243"/>
-      <c r="AO5" s="244"/>
-      <c r="AP5" s="261" t="s">
+      <c r="Z5" s="273"/>
+      <c r="AA5" s="273"/>
+      <c r="AB5" s="273"/>
+      <c r="AC5" s="273"/>
+      <c r="AD5" s="273"/>
+      <c r="AE5" s="273"/>
+      <c r="AF5" s="273"/>
+      <c r="AG5" s="273"/>
+      <c r="AH5" s="273"/>
+      <c r="AI5" s="273"/>
+      <c r="AJ5" s="273"/>
+      <c r="AK5" s="273"/>
+      <c r="AL5" s="273"/>
+      <c r="AM5" s="273"/>
+      <c r="AN5" s="273"/>
+      <c r="AO5" s="274"/>
+      <c r="AP5" s="252" t="s">
         <v>16</v>
       </c>
-      <c r="AQ5" s="261" t="s">
+      <c r="AQ5" s="252" t="s">
         <v>17</v>
       </c>
-      <c r="AR5" s="261" t="s">
+      <c r="AR5" s="252" t="s">
         <v>18</v>
       </c>
-      <c r="AS5" s="261" t="s">
+      <c r="AS5" s="252" t="s">
         <v>19</v>
       </c>
-      <c r="AT5" s="261" t="s">
+      <c r="AT5" s="252" t="s">
         <v>20</v>
       </c>
-      <c r="AU5" s="261" t="s">
+      <c r="AU5" s="252" t="s">
         <v>21</v>
       </c>
-      <c r="AV5" s="261" t="s">
+      <c r="AV5" s="252" t="s">
         <v>22</v>
       </c>
-      <c r="AW5" s="261" t="s">
+      <c r="AW5" s="252" t="s">
         <v>23</v>
       </c>
-      <c r="AX5" s="261" t="s">
+      <c r="AX5" s="252" t="s">
         <v>24</v>
       </c>
-      <c r="AY5" s="268" t="s">
+      <c r="AY5" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ5" s="243"/>
-      <c r="BA5" s="243"/>
-      <c r="BB5" s="243"/>
-      <c r="BC5" s="243"/>
-      <c r="BD5" s="243"/>
-      <c r="BE5" s="243"/>
-      <c r="BF5" s="243"/>
-      <c r="BG5" s="243"/>
-      <c r="BH5" s="243"/>
-      <c r="BI5" s="243"/>
-      <c r="BJ5" s="243"/>
-      <c r="BK5" s="243"/>
-      <c r="BL5" s="243"/>
-      <c r="BM5" s="243"/>
-      <c r="BN5" s="243"/>
-      <c r="BO5" s="243"/>
-      <c r="BP5" s="244"/>
-      <c r="BQ5" s="280" t="s">
+      <c r="AZ5" s="273"/>
+      <c r="BA5" s="273"/>
+      <c r="BB5" s="273"/>
+      <c r="BC5" s="273"/>
+      <c r="BD5" s="273"/>
+      <c r="BE5" s="273"/>
+      <c r="BF5" s="273"/>
+      <c r="BG5" s="273"/>
+      <c r="BH5" s="273"/>
+      <c r="BI5" s="273"/>
+      <c r="BJ5" s="273"/>
+      <c r="BK5" s="273"/>
+      <c r="BL5" s="273"/>
+      <c r="BM5" s="273"/>
+      <c r="BN5" s="273"/>
+      <c r="BO5" s="273"/>
+      <c r="BP5" s="274"/>
+      <c r="BQ5" s="253" t="s">
         <v>26</v>
       </c>
       <c r="BR5" s="254"/>
-      <c r="BS5" s="268" t="s">
+      <c r="BS5" s="261" t="s">
         <v>143</v>
       </c>
-      <c r="BT5" s="268" t="s">
+      <c r="BT5" s="261" t="s">
         <v>27</v>
       </c>
-      <c r="BU5" s="281" t="s">
+      <c r="BU5" s="257" t="s">
         <v>28</v>
       </c>
-      <c r="BW5" s="262" t="s">
+      <c r="BW5" s="286" t="s">
         <v>29</v>
       </c>
-      <c r="BX5" s="252" t="s">
+      <c r="BX5" s="279" t="s">
         <v>30</v>
       </c>
-      <c r="BY5" s="253"/>
-      <c r="BZ5" s="253"/>
+      <c r="BY5" s="280"/>
+      <c r="BZ5" s="280"/>
       <c r="CA5" s="254"/>
-      <c r="CB5" s="266" t="s">
+      <c r="CB5" s="272" t="s">
         <v>31</v>
       </c>
-      <c r="CC5" s="276" t="s">
+      <c r="CC5" s="244" t="s">
         <v>32</v>
       </c>
-      <c r="CD5" s="276" t="s">
+      <c r="CD5" s="244" t="s">
         <v>33</v>
       </c>
       <c r="CH5" s="142"/>
       <c r="CI5" s="143"/>
     </row>
     <row r="6" spans="1:87" s="141" customFormat="1">
-      <c r="A6" s="248"/>
-      <c r="B6" s="248"/>
-      <c r="C6" s="248"/>
-      <c r="D6" s="248"/>
-      <c r="E6" s="248"/>
-      <c r="F6" s="248"/>
-      <c r="G6" s="248"/>
-      <c r="H6" s="248"/>
-      <c r="I6" s="248"/>
-      <c r="J6" s="248"/>
-      <c r="K6" s="286" t="s">
+      <c r="A6" s="245"/>
+      <c r="B6" s="245"/>
+      <c r="C6" s="245"/>
+      <c r="D6" s="245"/>
+      <c r="E6" s="245"/>
+      <c r="F6" s="245"/>
+      <c r="G6" s="245"/>
+      <c r="H6" s="245"/>
+      <c r="I6" s="245"/>
+      <c r="J6" s="245"/>
+      <c r="K6" s="288" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="286" t="s">
+      <c r="L6" s="288" t="s">
         <v>35</v>
       </c>
-      <c r="M6" s="286" t="s">
+      <c r="M6" s="288" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="286" t="s">
+      <c r="N6" s="288" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="286" t="s">
+      <c r="O6" s="288" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="286" t="s">
+      <c r="P6" s="288" t="s">
         <v>39</v>
       </c>
-      <c r="Q6" s="286" t="s">
+      <c r="Q6" s="288" t="s">
         <v>40</v>
       </c>
-      <c r="R6" s="286" t="s">
+      <c r="R6" s="288" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="286" t="s">
+      <c r="S6" s="288" t="s">
         <v>42</v>
       </c>
-      <c r="T6" s="286" t="s">
+      <c r="T6" s="288" t="s">
         <v>43</v>
       </c>
-      <c r="U6" s="286" t="s">
+      <c r="U6" s="288" t="s">
         <v>44</v>
       </c>
-      <c r="V6" s="289" t="s">
+      <c r="V6" s="295" t="s">
         <v>45</v>
       </c>
       <c r="W6" s="254"/>
-      <c r="X6" s="286" t="s">
+      <c r="X6" s="288" t="s">
         <v>46</v>
       </c>
-      <c r="Y6" s="261" t="s">
+      <c r="Y6" s="252" t="s">
         <v>47</v>
       </c>
-      <c r="Z6" s="261" t="s">
+      <c r="Z6" s="252" t="s">
         <v>48</v>
       </c>
-      <c r="AA6" s="261" t="s">
+      <c r="AA6" s="252" t="s">
         <v>49</v>
       </c>
-      <c r="AB6" s="261" t="s">
+      <c r="AB6" s="252" t="s">
         <v>50</v>
       </c>
-      <c r="AC6" s="287" t="s">
+      <c r="AC6" s="289" t="s">
         <v>51</v>
       </c>
-      <c r="AD6" s="287" t="s">
+      <c r="AD6" s="289" t="s">
         <v>144</v>
       </c>
-      <c r="AE6" s="287" t="s">
+      <c r="AE6" s="289" t="s">
         <v>53</v>
       </c>
-      <c r="AF6" s="287" t="s">
+      <c r="AF6" s="289" t="s">
         <v>54</v>
       </c>
-      <c r="AG6" s="261" t="s">
+      <c r="AG6" s="252" t="s">
         <v>55</v>
       </c>
-      <c r="AH6" s="287" t="s">
+      <c r="AH6" s="289" t="s">
         <v>56</v>
       </c>
-      <c r="AI6" s="287" t="s">
+      <c r="AI6" s="289" t="s">
         <v>57</v>
       </c>
-      <c r="AJ6" s="261" t="s">
+      <c r="AJ6" s="252" t="s">
         <v>58</v>
       </c>
-      <c r="AK6" s="283" t="s">
+      <c r="AK6" s="249" t="s">
         <v>59</v>
       </c>
-      <c r="AL6" s="261" t="s">
+      <c r="AL6" s="252" t="s">
         <v>60</v>
       </c>
-      <c r="AM6" s="261" t="s">
+      <c r="AM6" s="252" t="s">
         <v>61</v>
       </c>
-      <c r="AN6" s="269" t="s">
+      <c r="AN6" s="275" t="s">
         <v>62</v>
       </c>
-      <c r="AO6" s="261" t="s">
+      <c r="AO6" s="252" t="s">
         <v>63</v>
       </c>
-      <c r="AP6" s="248"/>
-      <c r="AQ6" s="248"/>
-      <c r="AR6" s="248"/>
-      <c r="AS6" s="248"/>
-      <c r="AT6" s="248"/>
-      <c r="AU6" s="248"/>
-      <c r="AV6" s="248"/>
-      <c r="AW6" s="248"/>
-      <c r="AX6" s="248"/>
-      <c r="AY6" s="268" t="s">
+      <c r="AP6" s="245"/>
+      <c r="AQ6" s="245"/>
+      <c r="AR6" s="245"/>
+      <c r="AS6" s="245"/>
+      <c r="AT6" s="245"/>
+      <c r="AU6" s="245"/>
+      <c r="AV6" s="245"/>
+      <c r="AW6" s="245"/>
+      <c r="AX6" s="245"/>
+      <c r="AY6" s="261" t="s">
         <v>25</v>
       </c>
-      <c r="AZ6" s="243"/>
-      <c r="BA6" s="243"/>
-      <c r="BB6" s="243"/>
-      <c r="BC6" s="243"/>
-      <c r="BD6" s="243"/>
-      <c r="BE6" s="243"/>
-      <c r="BF6" s="243"/>
-      <c r="BG6" s="243"/>
-      <c r="BH6" s="243"/>
-      <c r="BI6" s="243"/>
-      <c r="BJ6" s="244"/>
-      <c r="BK6" s="268" t="s">
+      <c r="AZ6" s="273"/>
+      <c r="BA6" s="273"/>
+      <c r="BB6" s="273"/>
+      <c r="BC6" s="273"/>
+      <c r="BD6" s="273"/>
+      <c r="BE6" s="273"/>
+      <c r="BF6" s="273"/>
+      <c r="BG6" s="273"/>
+      <c r="BH6" s="273"/>
+      <c r="BI6" s="273"/>
+      <c r="BJ6" s="274"/>
+      <c r="BK6" s="261" t="s">
         <v>64</v>
       </c>
-      <c r="BL6" s="243"/>
-      <c r="BM6" s="243"/>
-      <c r="BN6" s="243"/>
-      <c r="BO6" s="243"/>
-      <c r="BP6" s="244"/>
-      <c r="BQ6" s="265" t="s">
+      <c r="BL6" s="273"/>
+      <c r="BM6" s="273"/>
+      <c r="BN6" s="273"/>
+      <c r="BO6" s="273"/>
+      <c r="BP6" s="274"/>
+      <c r="BQ6" s="259" t="s">
         <v>65</v>
       </c>
-      <c r="BR6" s="265" t="s">
+      <c r="BR6" s="259" t="s">
         <v>66</v>
       </c>
-      <c r="BS6" s="248"/>
-      <c r="BT6" s="248"/>
-      <c r="BU6" s="255"/>
-      <c r="BW6" s="257"/>
-      <c r="BX6" s="255"/>
+      <c r="BS6" s="245"/>
+      <c r="BT6" s="245"/>
+      <c r="BU6" s="250"/>
+      <c r="BW6" s="282"/>
+      <c r="BX6" s="250"/>
       <c r="BY6" s="292"/>
       <c r="BZ6" s="292"/>
-      <c r="CA6" s="257"/>
-      <c r="CB6" s="248"/>
-      <c r="CC6" s="248"/>
-      <c r="CD6" s="248"/>
+      <c r="CA6" s="282"/>
+      <c r="CB6" s="245"/>
+      <c r="CC6" s="245"/>
+      <c r="CD6" s="245"/>
       <c r="CH6" s="142"/>
       <c r="CI6" s="143"/>
     </row>
     <row r="7" spans="1:87" s="141" customFormat="1" ht="12">
-      <c r="A7" s="248"/>
-      <c r="B7" s="248"/>
-      <c r="C7" s="248"/>
-      <c r="D7" s="248"/>
-      <c r="E7" s="248"/>
-      <c r="F7" s="248"/>
-      <c r="G7" s="248"/>
-      <c r="H7" s="248"/>
-      <c r="I7" s="248"/>
-      <c r="J7" s="248"/>
-      <c r="K7" s="248"/>
-      <c r="L7" s="248"/>
-      <c r="M7" s="248"/>
-      <c r="N7" s="248"/>
-      <c r="O7" s="248"/>
-      <c r="P7" s="248"/>
-      <c r="Q7" s="248"/>
-      <c r="R7" s="248"/>
-      <c r="S7" s="248"/>
-      <c r="T7" s="248"/>
-      <c r="U7" s="248"/>
-      <c r="V7" s="282"/>
-      <c r="W7" s="285"/>
-      <c r="X7" s="248"/>
-      <c r="Y7" s="248"/>
-      <c r="Z7" s="248"/>
-      <c r="AA7" s="248"/>
-      <c r="AB7" s="248"/>
-      <c r="AC7" s="248"/>
-      <c r="AD7" s="248"/>
-      <c r="AE7" s="248"/>
-      <c r="AF7" s="248"/>
-      <c r="AG7" s="248"/>
-      <c r="AH7" s="248"/>
-      <c r="AI7" s="248"/>
-      <c r="AJ7" s="248"/>
-      <c r="AK7" s="255"/>
-      <c r="AL7" s="248"/>
-      <c r="AM7" s="248"/>
-      <c r="AN7" s="248"/>
-      <c r="AO7" s="248"/>
-      <c r="AP7" s="248"/>
-      <c r="AQ7" s="248"/>
-      <c r="AR7" s="248"/>
-      <c r="AS7" s="248"/>
-      <c r="AT7" s="248"/>
-      <c r="AU7" s="248"/>
-      <c r="AV7" s="248"/>
-      <c r="AW7" s="248"/>
-      <c r="AX7" s="248"/>
+      <c r="A7" s="245"/>
+      <c r="B7" s="245"/>
+      <c r="C7" s="245"/>
+      <c r="D7" s="245"/>
+      <c r="E7" s="245"/>
+      <c r="F7" s="245"/>
+      <c r="G7" s="245"/>
+      <c r="H7" s="245"/>
+      <c r="I7" s="245"/>
+      <c r="J7" s="245"/>
+      <c r="K7" s="245"/>
+      <c r="L7" s="245"/>
+      <c r="M7" s="245"/>
+      <c r="N7" s="245"/>
+      <c r="O7" s="245"/>
+      <c r="P7" s="245"/>
+      <c r="Q7" s="245"/>
+      <c r="R7" s="245"/>
+      <c r="S7" s="245"/>
+      <c r="T7" s="245"/>
+      <c r="U7" s="245"/>
+      <c r="V7" s="251"/>
+      <c r="W7" s="264"/>
+      <c r="X7" s="245"/>
+      <c r="Y7" s="245"/>
+      <c r="Z7" s="245"/>
+      <c r="AA7" s="245"/>
+      <c r="AB7" s="245"/>
+      <c r="AC7" s="245"/>
+      <c r="AD7" s="245"/>
+      <c r="AE7" s="245"/>
+      <c r="AF7" s="245"/>
+      <c r="AG7" s="245"/>
+      <c r="AH7" s="245"/>
+      <c r="AI7" s="245"/>
+      <c r="AJ7" s="245"/>
+      <c r="AK7" s="250"/>
+      <c r="AL7" s="245"/>
+      <c r="AM7" s="245"/>
+      <c r="AN7" s="245"/>
+      <c r="AO7" s="245"/>
+      <c r="AP7" s="245"/>
+      <c r="AQ7" s="245"/>
+      <c r="AR7" s="245"/>
+      <c r="AS7" s="245"/>
+      <c r="AT7" s="245"/>
+      <c r="AU7" s="245"/>
+      <c r="AV7" s="245"/>
+      <c r="AW7" s="245"/>
+      <c r="AX7" s="245"/>
       <c r="AY7" s="101" t="s">
         <v>67</v>
       </c>
@@ -18583,122 +18743,122 @@
       <c r="BA7" s="101" t="s">
         <v>69</v>
       </c>
-      <c r="BB7" s="268" t="s">
+      <c r="BB7" s="261" t="s">
         <v>70</v>
       </c>
-      <c r="BC7" s="245" t="s">
+      <c r="BC7" s="260" t="s">
         <v>71</v>
       </c>
-      <c r="BD7" s="245" t="s">
+      <c r="BD7" s="260" t="s">
         <v>72</v>
       </c>
-      <c r="BE7" s="245" t="s">
+      <c r="BE7" s="260" t="s">
         <v>145</v>
       </c>
-      <c r="BF7" s="245" t="s">
+      <c r="BF7" s="260" t="s">
         <v>74</v>
       </c>
-      <c r="BG7" s="245" t="s">
+      <c r="BG7" s="260" t="s">
         <v>75</v>
       </c>
-      <c r="BH7" s="245" t="s">
+      <c r="BH7" s="260" t="s">
         <v>76</v>
       </c>
-      <c r="BI7" s="245" t="s">
+      <c r="BI7" s="260" t="s">
         <v>79</v>
       </c>
-      <c r="BJ7" s="264" t="s">
+      <c r="BJ7" s="287" t="s">
         <v>80</v>
       </c>
-      <c r="BK7" s="245" t="s">
+      <c r="BK7" s="260" t="s">
         <v>81</v>
       </c>
-      <c r="BL7" s="268" t="s">
+      <c r="BL7" s="261" t="s">
         <v>82</v>
       </c>
-      <c r="BM7" s="245" t="s">
+      <c r="BM7" s="260" t="s">
         <v>83</v>
       </c>
-      <c r="BN7" s="268" t="s">
+      <c r="BN7" s="261" t="s">
         <v>84</v>
       </c>
-      <c r="BO7" s="268" t="s">
+      <c r="BO7" s="261" t="s">
         <v>146</v>
       </c>
-      <c r="BP7" s="268" t="s">
+      <c r="BP7" s="261" t="s">
         <v>85</v>
       </c>
-      <c r="BQ7" s="248"/>
-      <c r="BR7" s="248"/>
-      <c r="BS7" s="248"/>
-      <c r="BT7" s="248"/>
-      <c r="BU7" s="255"/>
-      <c r="BW7" s="257"/>
-      <c r="BX7" s="258"/>
-      <c r="BY7" s="259"/>
-      <c r="BZ7" s="259"/>
-      <c r="CA7" s="260"/>
-      <c r="CB7" s="248"/>
-      <c r="CC7" s="248"/>
-      <c r="CD7" s="248"/>
+      <c r="BQ7" s="245"/>
+      <c r="BR7" s="245"/>
+      <c r="BS7" s="245"/>
+      <c r="BT7" s="245"/>
+      <c r="BU7" s="250"/>
+      <c r="BW7" s="282"/>
+      <c r="BX7" s="283"/>
+      <c r="BY7" s="284"/>
+      <c r="BZ7" s="284"/>
+      <c r="CA7" s="285"/>
+      <c r="CB7" s="245"/>
+      <c r="CC7" s="245"/>
+      <c r="CD7" s="245"/>
       <c r="CH7" s="142"/>
       <c r="CI7" s="143"/>
     </row>
     <row r="8" spans="1:87" s="141" customFormat="1" ht="22.5" customHeight="1">
-      <c r="A8" s="246"/>
-      <c r="B8" s="246"/>
-      <c r="C8" s="246"/>
-      <c r="D8" s="246"/>
-      <c r="E8" s="246"/>
-      <c r="F8" s="246"/>
-      <c r="G8" s="246"/>
-      <c r="H8" s="246"/>
-      <c r="I8" s="246"/>
-      <c r="J8" s="246"/>
-      <c r="K8" s="246"/>
-      <c r="L8" s="246"/>
-      <c r="M8" s="246"/>
-      <c r="N8" s="246"/>
-      <c r="O8" s="246"/>
-      <c r="P8" s="246"/>
-      <c r="Q8" s="246"/>
-      <c r="R8" s="246"/>
-      <c r="S8" s="246"/>
-      <c r="T8" s="246"/>
-      <c r="U8" s="246"/>
+      <c r="A8" s="248"/>
+      <c r="B8" s="248"/>
+      <c r="C8" s="248"/>
+      <c r="D8" s="248"/>
+      <c r="E8" s="248"/>
+      <c r="F8" s="248"/>
+      <c r="G8" s="248"/>
+      <c r="H8" s="248"/>
+      <c r="I8" s="248"/>
+      <c r="J8" s="248"/>
+      <c r="K8" s="248"/>
+      <c r="L8" s="248"/>
+      <c r="M8" s="248"/>
+      <c r="N8" s="248"/>
+      <c r="O8" s="248"/>
+      <c r="P8" s="248"/>
+      <c r="Q8" s="248"/>
+      <c r="R8" s="248"/>
+      <c r="S8" s="248"/>
+      <c r="T8" s="248"/>
+      <c r="U8" s="248"/>
       <c r="V8" s="145" t="s">
         <v>86</v>
       </c>
       <c r="W8" s="145" t="s">
         <v>87</v>
       </c>
-      <c r="X8" s="246"/>
-      <c r="Y8" s="246"/>
-      <c r="Z8" s="246"/>
-      <c r="AA8" s="246"/>
-      <c r="AB8" s="246"/>
-      <c r="AC8" s="246"/>
-      <c r="AD8" s="246"/>
-      <c r="AE8" s="246"/>
-      <c r="AF8" s="246"/>
-      <c r="AG8" s="246"/>
-      <c r="AH8" s="246"/>
-      <c r="AI8" s="246"/>
-      <c r="AJ8" s="246"/>
-      <c r="AK8" s="282"/>
-      <c r="AL8" s="246"/>
-      <c r="AM8" s="246"/>
-      <c r="AN8" s="246"/>
-      <c r="AO8" s="246"/>
-      <c r="AP8" s="246"/>
-      <c r="AQ8" s="246"/>
-      <c r="AR8" s="246"/>
-      <c r="AS8" s="246"/>
-      <c r="AT8" s="246"/>
-      <c r="AU8" s="246"/>
-      <c r="AV8" s="246"/>
-      <c r="AW8" s="246"/>
-      <c r="AX8" s="246"/>
+      <c r="X8" s="248"/>
+      <c r="Y8" s="248"/>
+      <c r="Z8" s="248"/>
+      <c r="AA8" s="248"/>
+      <c r="AB8" s="248"/>
+      <c r="AC8" s="248"/>
+      <c r="AD8" s="248"/>
+      <c r="AE8" s="248"/>
+      <c r="AF8" s="248"/>
+      <c r="AG8" s="248"/>
+      <c r="AH8" s="248"/>
+      <c r="AI8" s="248"/>
+      <c r="AJ8" s="248"/>
+      <c r="AK8" s="251"/>
+      <c r="AL8" s="248"/>
+      <c r="AM8" s="248"/>
+      <c r="AN8" s="248"/>
+      <c r="AO8" s="248"/>
+      <c r="AP8" s="248"/>
+      <c r="AQ8" s="248"/>
+      <c r="AR8" s="248"/>
+      <c r="AS8" s="248"/>
+      <c r="AT8" s="248"/>
+      <c r="AU8" s="248"/>
+      <c r="AV8" s="248"/>
+      <c r="AW8" s="248"/>
+      <c r="AX8" s="248"/>
       <c r="AY8" s="102" t="s">
         <v>88</v>
       </c>
@@ -18708,27 +18868,27 @@
       <c r="BA8" s="102" t="s">
         <v>90</v>
       </c>
-      <c r="BB8" s="246"/>
-      <c r="BC8" s="246"/>
-      <c r="BD8" s="246"/>
-      <c r="BE8" s="246"/>
-      <c r="BF8" s="246"/>
-      <c r="BG8" s="246"/>
-      <c r="BH8" s="246"/>
-      <c r="BI8" s="246"/>
-      <c r="BJ8" s="246"/>
-      <c r="BK8" s="246"/>
-      <c r="BL8" s="246"/>
-      <c r="BM8" s="246"/>
-      <c r="BN8" s="246"/>
-      <c r="BO8" s="246"/>
-      <c r="BP8" s="246"/>
-      <c r="BQ8" s="246"/>
-      <c r="BR8" s="246"/>
-      <c r="BS8" s="246"/>
-      <c r="BT8" s="246"/>
-      <c r="BU8" s="282"/>
-      <c r="BW8" s="260"/>
+      <c r="BB8" s="248"/>
+      <c r="BC8" s="248"/>
+      <c r="BD8" s="248"/>
+      <c r="BE8" s="248"/>
+      <c r="BF8" s="248"/>
+      <c r="BG8" s="248"/>
+      <c r="BH8" s="248"/>
+      <c r="BI8" s="248"/>
+      <c r="BJ8" s="248"/>
+      <c r="BK8" s="248"/>
+      <c r="BL8" s="248"/>
+      <c r="BM8" s="248"/>
+      <c r="BN8" s="248"/>
+      <c r="BO8" s="248"/>
+      <c r="BP8" s="248"/>
+      <c r="BQ8" s="248"/>
+      <c r="BR8" s="248"/>
+      <c r="BS8" s="248"/>
+      <c r="BT8" s="248"/>
+      <c r="BU8" s="251"/>
+      <c r="BW8" s="285"/>
       <c r="BX8" s="72" t="s">
         <v>91</v>
       </c>
@@ -18741,9 +18901,9 @@
       <c r="CA8" s="73" t="s">
         <v>94</v>
       </c>
-      <c r="CB8" s="267"/>
-      <c r="CC8" s="267"/>
-      <c r="CD8" s="267"/>
+      <c r="CB8" s="246"/>
+      <c r="CC8" s="246"/>
+      <c r="CD8" s="246"/>
       <c r="CF8" s="146"/>
       <c r="CH8" s="142"/>
       <c r="CI8" s="143"/>
@@ -20742,14 +20902,88 @@
       <c r="CG19" s="213"/>
       <c r="CI19" s="215"/>
     </row>
+    <row r="22" spans="1:87">
+      <c r="C22" s="303" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:87">
+      <c r="C23" s="302"/>
+    </row>
     <row r="25" spans="1:87" ht="17">
-      <c r="G25" s="299" t="s">
+      <c r="G25" s="242" t="s">
         <v>153</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A9:CI14" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <mergeCells count="82">
+    <mergeCell ref="BC7:BC8"/>
+    <mergeCell ref="AE6:AE8"/>
+    <mergeCell ref="CB5:CB8"/>
+    <mergeCell ref="BT5:BT8"/>
+    <mergeCell ref="AL6:AL8"/>
+    <mergeCell ref="P6:P8"/>
+    <mergeCell ref="BB7:BB8"/>
+    <mergeCell ref="BD7:BD8"/>
+    <mergeCell ref="BF7:BF8"/>
+    <mergeCell ref="BH7:BH8"/>
+    <mergeCell ref="S6:S8"/>
+    <mergeCell ref="AS5:AS8"/>
+    <mergeCell ref="BQ5:BR5"/>
+    <mergeCell ref="BK7:BK8"/>
+    <mergeCell ref="BK6:BP6"/>
+    <mergeCell ref="BN7:BN8"/>
+    <mergeCell ref="BP7:BP8"/>
+    <mergeCell ref="AM6:AM8"/>
+    <mergeCell ref="D5:D8"/>
+    <mergeCell ref="X6:X8"/>
+    <mergeCell ref="AV5:AV8"/>
+    <mergeCell ref="AX5:AX8"/>
+    <mergeCell ref="V6:W7"/>
+    <mergeCell ref="Y6:Y8"/>
+    <mergeCell ref="N6:N8"/>
+    <mergeCell ref="F5:F8"/>
+    <mergeCell ref="AP5:AP8"/>
+    <mergeCell ref="AB6:AB8"/>
+    <mergeCell ref="M6:M8"/>
+    <mergeCell ref="AH6:AH8"/>
+    <mergeCell ref="AJ6:AJ8"/>
+    <mergeCell ref="T6:T8"/>
+    <mergeCell ref="Q6:Q8"/>
+    <mergeCell ref="AC6:AC8"/>
+    <mergeCell ref="A3:BU3"/>
+    <mergeCell ref="E5:E8"/>
+    <mergeCell ref="K6:K8"/>
+    <mergeCell ref="BS5:BS8"/>
+    <mergeCell ref="O6:O8"/>
+    <mergeCell ref="G5:G8"/>
+    <mergeCell ref="I5:I8"/>
+    <mergeCell ref="AQ5:AQ8"/>
+    <mergeCell ref="R6:R8"/>
+    <mergeCell ref="B5:B8"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="C5:C8"/>
+    <mergeCell ref="AU5:AU8"/>
+    <mergeCell ref="AK6:AK8"/>
+    <mergeCell ref="BI7:BI8"/>
+    <mergeCell ref="K5:X5"/>
+    <mergeCell ref="BX5:CA7"/>
+    <mergeCell ref="U6:U8"/>
+    <mergeCell ref="AY6:BJ6"/>
+    <mergeCell ref="AG6:AG8"/>
+    <mergeCell ref="BE7:BE8"/>
+    <mergeCell ref="BQ6:BQ8"/>
+    <mergeCell ref="BG7:BG8"/>
+    <mergeCell ref="AD6:AD8"/>
+    <mergeCell ref="AF6:AF8"/>
+    <mergeCell ref="AO6:AO8"/>
+    <mergeCell ref="Y5:AO5"/>
+    <mergeCell ref="AN6:AN8"/>
+    <mergeCell ref="AR5:AR8"/>
+    <mergeCell ref="AA6:AA8"/>
+    <mergeCell ref="BO7:BO8"/>
+    <mergeCell ref="AY5:BP5"/>
     <mergeCell ref="BW3:CB4"/>
     <mergeCell ref="CC5:CC8"/>
     <mergeCell ref="H5:H8"/>
@@ -20766,72 +21000,6 @@
     <mergeCell ref="AI6:AI8"/>
     <mergeCell ref="BU5:BU8"/>
     <mergeCell ref="BW5:BW8"/>
-    <mergeCell ref="BX5:CA7"/>
-    <mergeCell ref="U6:U8"/>
-    <mergeCell ref="AY6:BJ6"/>
-    <mergeCell ref="AG6:AG8"/>
-    <mergeCell ref="BE7:BE8"/>
-    <mergeCell ref="BQ6:BQ8"/>
-    <mergeCell ref="BG7:BG8"/>
-    <mergeCell ref="AD6:AD8"/>
-    <mergeCell ref="AF6:AF8"/>
-    <mergeCell ref="A3:BU3"/>
-    <mergeCell ref="E5:E8"/>
-    <mergeCell ref="K6:K8"/>
-    <mergeCell ref="BS5:BS8"/>
-    <mergeCell ref="O6:O8"/>
-    <mergeCell ref="G5:G8"/>
-    <mergeCell ref="I5:I8"/>
-    <mergeCell ref="AQ5:AQ8"/>
-    <mergeCell ref="R6:R8"/>
-    <mergeCell ref="B5:B8"/>
-    <mergeCell ref="A5:A8"/>
-    <mergeCell ref="C5:C8"/>
-    <mergeCell ref="AU5:AU8"/>
-    <mergeCell ref="AK6:AK8"/>
-    <mergeCell ref="BI7:BI8"/>
-    <mergeCell ref="K5:X5"/>
-    <mergeCell ref="AO6:AO8"/>
-    <mergeCell ref="Y5:AO5"/>
-    <mergeCell ref="AN6:AN8"/>
-    <mergeCell ref="AR5:AR8"/>
-    <mergeCell ref="AA6:AA8"/>
-    <mergeCell ref="D5:D8"/>
-    <mergeCell ref="X6:X8"/>
-    <mergeCell ref="AV5:AV8"/>
-    <mergeCell ref="AX5:AX8"/>
-    <mergeCell ref="V6:W7"/>
-    <mergeCell ref="Y6:Y8"/>
-    <mergeCell ref="CB5:CB8"/>
-    <mergeCell ref="BT5:BT8"/>
-    <mergeCell ref="AL6:AL8"/>
-    <mergeCell ref="P6:P8"/>
-    <mergeCell ref="BB7:BB8"/>
-    <mergeCell ref="BD7:BD8"/>
-    <mergeCell ref="BF7:BF8"/>
-    <mergeCell ref="BH7:BH8"/>
-    <mergeCell ref="S6:S8"/>
-    <mergeCell ref="AS5:AS8"/>
-    <mergeCell ref="BQ5:BR5"/>
-    <mergeCell ref="BK7:BK8"/>
-    <mergeCell ref="BK6:BP6"/>
-    <mergeCell ref="BN7:BN8"/>
-    <mergeCell ref="BP7:BP8"/>
-    <mergeCell ref="AM6:AM8"/>
-    <mergeCell ref="N6:N8"/>
-    <mergeCell ref="F5:F8"/>
-    <mergeCell ref="AP5:AP8"/>
-    <mergeCell ref="BO7:BO8"/>
-    <mergeCell ref="AB6:AB8"/>
-    <mergeCell ref="AY5:BP5"/>
-    <mergeCell ref="M6:M8"/>
-    <mergeCell ref="AH6:AH8"/>
-    <mergeCell ref="AJ6:AJ8"/>
-    <mergeCell ref="T6:T8"/>
-    <mergeCell ref="Q6:Q8"/>
-    <mergeCell ref="AC6:AC8"/>
-    <mergeCell ref="BC7:BC8"/>
-    <mergeCell ref="AE6:AE8"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:B9 B12:B16 B20:B1048576 C9:BU9 D10:F10 J10:BI10 BK10:BU10 BW9:CD10">
     <cfRule type="duplicateValues" dxfId="6" priority="68"/>

</xml_diff>